<commit_message>
fixed: formatted itin schedule
</commit_message>
<xml_diff>
--- a/database/horarios/HORARIO_ITIJ_202551.xlsx
+++ b/database/horarios/HORARIO_ITIJ_202551.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johng\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johng\ESPE\Aplicaciones distribuidas\Proyecto\api-shedsync\database\horarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7A2AAE-D7EF-42C6-A4C6-921E01B7E2D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF9040F-469A-4DE5-89C2-E0842411D197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="1380" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
@@ -2560,7 +2560,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -2593,13 +2593,6 @@
       <sz val="8.5"/>
       <color rgb="FF000000"/>
       <name val="Arial MT"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="6.5"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
@@ -2892,16 +2885,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2911,79 +2901,73 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2992,107 +2976,128 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3100,28 +3105,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3428,13 +3412,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J80"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="10.6640625" customWidth="1"/>
-    <col min="2" max="2" width="8.5" customWidth="1"/>
-    <col min="3" max="3" width="52.1640625" customWidth="1"/>
-    <col min="4" max="4" width="6.5" customWidth="1"/>
+    <col min="2" max="3" width="8.5" customWidth="1"/>
+    <col min="4" max="4" width="52.1640625" customWidth="1"/>
     <col min="5" max="5" width="11.5" customWidth="1"/>
     <col min="6" max="6" width="13.33203125" customWidth="1"/>
     <col min="7" max="7" width="12.5" customWidth="1"/>
@@ -3444,86 +3427,86 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21.75" customHeight="1">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="34" t="s">
         <v>179</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
     </row>
     <row r="2" spans="1:10" ht="15.75">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="36" t="s">
         <v>180</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
     </row>
     <row r="3" spans="1:10" ht="24.75" customHeight="1">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="66" t="s">
         <v>181</v>
       </c>
-      <c r="B3" s="33"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
-      <c r="J3" s="33"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
     </row>
     <row r="4" spans="1:10" ht="25.7" customHeight="1">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="35"/>
-      <c r="I4" s="35"/>
-      <c r="J4" s="36"/>
+      <c r="B4" s="39"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="39"/>
+      <c r="H4" s="39"/>
+      <c r="I4" s="39"/>
+      <c r="J4" s="40"/>
     </row>
     <row r="5" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="41" t="s">
+      <c r="C5" s="30"/>
+      <c r="D5" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="43" t="s">
+      <c r="E5" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="44"/>
-      <c r="J5" s="45"/>
+      <c r="F5" s="48"/>
+      <c r="G5" s="48"/>
+      <c r="H5" s="48"/>
+      <c r="I5" s="48"/>
+      <c r="J5" s="49"/>
     </row>
     <row r="6" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A6" s="38"/>
-      <c r="B6" s="40"/>
-      <c r="C6" s="42"/>
-      <c r="D6" s="2"/>
+      <c r="A6" s="54"/>
+      <c r="B6" s="44"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="56"/>
       <c r="E6" s="1" t="s">
         <v>5</v>
       </c>
@@ -3539,413 +3522,385 @@
       <c r="I6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A7" s="46" t="s">
+      <c r="A7" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="3">
         <v>31033</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="3"/>
+      <c r="D7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="6">
+      <c r="E7" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="6"/>
+      <c r="G7" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="18.600000000000001" customHeight="1">
+      <c r="A8" s="60"/>
+      <c r="B8" s="3">
+        <v>29767</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="6"/>
+      <c r="F8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="6"/>
+      <c r="H8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="18.600000000000001" customHeight="1">
+      <c r="A9" s="60"/>
+      <c r="B9" s="3">
+        <v>31036</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="6"/>
+      <c r="G9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="6"/>
+      <c r="I9" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="18.600000000000001" customHeight="1">
+      <c r="A10" s="60"/>
+      <c r="B10" s="3">
+        <v>30530</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="24.2" customHeight="1">
+      <c r="A11" s="60"/>
+      <c r="B11" s="3">
+        <v>30534</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I11" s="6"/>
+      <c r="J11" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="18.600000000000001" customHeight="1">
+      <c r="A12" s="60"/>
+      <c r="B12" s="3">
+        <v>31545</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="6"/>
+      <c r="F12" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="18.600000000000001" customHeight="1">
+      <c r="A13" s="64"/>
+      <c r="B13" s="13">
+        <v>28841</v>
+      </c>
+      <c r="C13" s="13"/>
+      <c r="D13" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="6"/>
+      <c r="F13" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="11.1" customHeight="1">
+      <c r="A14" s="14"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="15"/>
+    </row>
+    <row r="15" spans="1:10" ht="18.600000000000001" customHeight="1">
+      <c r="A15" s="63" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="3">
+        <v>31034</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" s="6"/>
+      <c r="F15" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G15" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="23.25" customHeight="1">
+      <c r="A16" s="60"/>
+      <c r="B16" s="3">
+        <v>30742</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G16" s="6"/>
+      <c r="H16" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="I16" s="6"/>
+      <c r="J16" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="18.600000000000001" customHeight="1">
+      <c r="A17" s="60"/>
+      <c r="B17" s="3">
+        <v>31037</v>
+      </c>
+      <c r="C17" s="3"/>
+      <c r="D17" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F17" s="6"/>
+      <c r="G17" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="H17" s="6"/>
+      <c r="I17" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="24.2" customHeight="1">
+      <c r="A18" s="60"/>
+      <c r="B18" s="3">
+        <v>31914</v>
+      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="J18" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="24.2" customHeight="1">
+      <c r="A19" s="60"/>
+      <c r="B19" s="3">
+        <v>30531</v>
+      </c>
+      <c r="C19" s="3"/>
+      <c r="D19" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="21.6" customHeight="1">
+      <c r="A20" s="60"/>
+      <c r="B20" s="3">
+        <v>31695</v>
+      </c>
+      <c r="C20" s="3"/>
+      <c r="D20" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="I20" s="6"/>
+      <c r="J20" s="7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="25.35" customHeight="1">
+      <c r="A21" s="60"/>
+      <c r="B21" s="13">
+        <v>31975</v>
+      </c>
+      <c r="C21" s="13"/>
+      <c r="D21" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="E21" s="6"/>
+      <c r="F21" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="J21" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="12.75" customHeight="1">
+      <c r="A22" s="65"/>
+      <c r="B22" s="65"/>
+      <c r="C22" s="65"/>
+      <c r="D22" s="65"/>
+      <c r="E22" s="65"/>
+      <c r="F22" s="65"/>
+      <c r="G22" s="65"/>
+      <c r="H22" s="65"/>
+      <c r="I22" s="65"/>
+      <c r="J22" s="65"/>
+    </row>
+    <row r="23" spans="1:10" ht="16.5" customHeight="1">
+      <c r="A23" s="38" t="s">
+        <v>57</v>
+      </c>
+      <c r="B23" s="39"/>
+      <c r="C23" s="39"/>
+      <c r="D23" s="39"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="39"/>
+      <c r="I23" s="39"/>
+      <c r="J23" s="40"/>
+    </row>
+    <row r="24" spans="1:10" ht="13.7" customHeight="1">
+      <c r="A24" s="53" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" s="43" t="s">
+        <v>2</v>
+      </c>
+      <c r="C24" s="30"/>
+      <c r="D24" s="55" t="s">
+        <v>3</v>
+      </c>
+      <c r="E24" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A8" s="47"/>
-      <c r="B8" s="4">
-        <v>29767</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="6">
-        <v>6</v>
-      </c>
-      <c r="E8" s="8"/>
-      <c r="F8" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G8" s="8"/>
-      <c r="H8" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="J8" s="9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A9" s="47"/>
-      <c r="B9" s="4">
-        <v>31036</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="6">
-        <v>6</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" s="8"/>
-      <c r="G9" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="8"/>
-      <c r="I9" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="J9" s="9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A10" s="47"/>
-      <c r="B10" s="4">
-        <v>30530</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="6">
-        <v>3</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="24.2" customHeight="1">
-      <c r="A11" s="47"/>
-      <c r="B11" s="4">
-        <v>30534</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" s="13">
-        <v>3</v>
-      </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I11" s="8"/>
-      <c r="J11" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A12" s="47"/>
-      <c r="B12" s="4">
-        <v>31545</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="6">
-        <v>4</v>
-      </c>
-      <c r="E12" s="8"/>
-      <c r="F12" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="J12" s="9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A13" s="48"/>
-      <c r="B13" s="16">
-        <v>28841</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" s="6">
-        <v>4</v>
-      </c>
-      <c r="E13" s="8"/>
-      <c r="F13" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="J13" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="11.1" customHeight="1">
-      <c r="A14" s="17"/>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="49"/>
-      <c r="E14" s="50"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-    </row>
-    <row r="15" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A15" s="46" t="s">
-        <v>35</v>
-      </c>
-      <c r="B15" s="4">
-        <v>31034</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15" s="6">
-        <v>4</v>
-      </c>
-      <c r="E15" s="8"/>
-      <c r="F15" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G15" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="23.25" customHeight="1">
-      <c r="A16" s="47"/>
-      <c r="B16" s="4">
-        <v>30742</v>
-      </c>
-      <c r="C16" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="D16" s="13">
-        <v>6</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G16" s="8"/>
-      <c r="H16" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="I16" s="8"/>
-      <c r="J16" s="14" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A17" s="47"/>
-      <c r="B17" s="4">
-        <v>31037</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="6">
-        <v>6</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F17" s="8"/>
-      <c r="G17" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="H17" s="8"/>
-      <c r="I17" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="J17" s="9" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="24.2" customHeight="1">
-      <c r="A18" s="47"/>
-      <c r="B18" s="4">
-        <v>31914</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="D18" s="13">
-        <v>3</v>
-      </c>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="J18" s="14" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="24.2" customHeight="1">
-      <c r="A19" s="47"/>
-      <c r="B19" s="4">
-        <v>30531</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="D19" s="13">
-        <v>3</v>
-      </c>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="14" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="21.6" customHeight="1">
-      <c r="A20" s="47"/>
-      <c r="B20" s="4">
-        <v>31695</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D20" s="6">
-        <v>4</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="I20" s="8"/>
-      <c r="J20" s="9" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="25.35" customHeight="1">
-      <c r="A21" s="47"/>
-      <c r="B21" s="16">
-        <v>31975</v>
-      </c>
-      <c r="C21" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="D21" s="13">
-        <v>4</v>
-      </c>
-      <c r="E21" s="8"/>
-      <c r="F21" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="J21" s="14" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="12.75" customHeight="1">
-      <c r="A22" s="51"/>
-      <c r="B22" s="51"/>
-      <c r="C22" s="51"/>
-      <c r="D22" s="51"/>
-      <c r="E22" s="51"/>
-      <c r="F22" s="51"/>
-      <c r="G22" s="51"/>
-      <c r="H22" s="51"/>
-      <c r="I22" s="51"/>
-      <c r="J22" s="51"/>
-    </row>
-    <row r="23" spans="1:10" ht="16.5" customHeight="1">
-      <c r="A23" s="34" t="s">
-        <v>57</v>
-      </c>
-      <c r="B23" s="35"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35"/>
-      <c r="G23" s="35"/>
-      <c r="H23" s="35"/>
-      <c r="I23" s="35"/>
-      <c r="J23" s="36"/>
-    </row>
-    <row r="24" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A24" s="37" t="s">
-        <v>1</v>
-      </c>
-      <c r="B24" s="39" t="s">
-        <v>2</v>
-      </c>
-      <c r="C24" s="41" t="s">
-        <v>3</v>
-      </c>
-      <c r="D24" s="2"/>
-      <c r="E24" s="43" t="s">
-        <v>4</v>
-      </c>
-      <c r="F24" s="44"/>
-      <c r="G24" s="44"/>
-      <c r="H24" s="44"/>
-      <c r="I24" s="44"/>
-      <c r="J24" s="45"/>
+      <c r="F24" s="48"/>
+      <c r="G24" s="48"/>
+      <c r="H24" s="48"/>
+      <c r="I24" s="48"/>
+      <c r="J24" s="49"/>
     </row>
     <row r="25" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A25" s="38"/>
-      <c r="B25" s="40"/>
-      <c r="C25" s="42"/>
-      <c r="D25" s="2"/>
+      <c r="A25" s="54"/>
+      <c r="B25" s="44"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="56"/>
       <c r="E25" s="1" t="s">
         <v>5</v>
       </c>
@@ -3961,277 +3916,261 @@
       <c r="I25" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J25" s="3" t="s">
+      <c r="J25" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="19.7" customHeight="1">
-      <c r="A26" s="46" t="s">
+      <c r="A26" s="63" t="s">
         <v>58</v>
       </c>
-      <c r="B26" s="4">
+      <c r="B26" s="3">
         <v>30744</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="3"/>
+      <c r="D26" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="6">
-        <v>6</v>
-      </c>
-      <c r="E26" s="7" t="s">
+      <c r="E26" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="F26" s="8"/>
-      <c r="G26" s="7" t="s">
+      <c r="F26" s="6"/>
+      <c r="G26" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="H26" s="7" t="s">
+      <c r="H26" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="I26" s="8"/>
-      <c r="J26" s="9" t="s">
+      <c r="I26" s="6"/>
+      <c r="J26" s="7" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="19.7" customHeight="1">
-      <c r="A27" s="47"/>
-      <c r="B27" s="4">
+      <c r="A27" s="60"/>
+      <c r="B27" s="3">
         <v>30743</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="3"/>
+      <c r="D27" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="D27" s="6">
-        <v>6</v>
-      </c>
-      <c r="E27" s="8"/>
-      <c r="F27" s="7" t="s">
+      <c r="E27" s="6"/>
+      <c r="F27" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="G27" s="7" t="s">
+      <c r="G27" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="H27" s="8"/>
-      <c r="I27" s="7" t="s">
+      <c r="H27" s="6"/>
+      <c r="I27" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="J27" s="9" t="s">
+      <c r="J27" s="7" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="19.7" customHeight="1">
-      <c r="A28" s="47"/>
-      <c r="B28" s="4">
+      <c r="A28" s="60"/>
+      <c r="B28" s="3">
         <v>31048</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="3"/>
+      <c r="D28" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D28" s="6">
+      <c r="E28" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F28" s="6"/>
+      <c r="G28" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="H28" s="6"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="5.25" customHeight="1">
+      <c r="A29" s="59"/>
+      <c r="B29" s="59"/>
+      <c r="C29" s="59"/>
+      <c r="D29" s="59"/>
+      <c r="E29" s="59"/>
+      <c r="F29" s="59"/>
+      <c r="G29" s="59"/>
+      <c r="H29" s="59"/>
+      <c r="I29" s="59"/>
+      <c r="J29" s="59"/>
+    </row>
+    <row r="30" spans="1:10" ht="19.7" customHeight="1">
+      <c r="A30" s="60" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" s="3">
+        <v>31051</v>
+      </c>
+      <c r="C30" s="3"/>
+      <c r="D30" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E30" s="6"/>
+      <c r="F30" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G30" s="6"/>
+      <c r="H30" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="I30" s="6"/>
+      <c r="J30" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="22.35" customHeight="1">
+      <c r="A31" s="60"/>
+      <c r="B31" s="17">
+        <v>31041</v>
+      </c>
+      <c r="C31" s="17"/>
+      <c r="D31" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E31" s="6"/>
+      <c r="F31" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="J31" s="18" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="22.35" customHeight="1">
+      <c r="A32" s="61" t="s">
+        <v>77</v>
+      </c>
+      <c r="B32" s="19">
+        <v>30745</v>
+      </c>
+      <c r="C32" s="19"/>
+      <c r="D32" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="E32" s="6"/>
+      <c r="F32" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="H32" s="6"/>
+      <c r="I32" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="J32" s="20" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="19.7" customHeight="1">
+      <c r="A33" s="61"/>
+      <c r="B33" s="3">
+        <v>31235</v>
+      </c>
+      <c r="C33" s="3"/>
+      <c r="D33" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E33" s="6"/>
+      <c r="F33" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="G33" s="6"/>
+      <c r="H33" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="I33" s="6"/>
+      <c r="J33" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="19.7" customHeight="1">
+      <c r="A34" s="61"/>
+      <c r="B34" s="17">
+        <v>31042</v>
+      </c>
+      <c r="C34" s="17"/>
+      <c r="D34" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+      <c r="I34" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="J34" s="7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="13.7" customHeight="1">
+      <c r="A35" s="21"/>
+      <c r="B35" s="62"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="37"/>
+      <c r="H35" s="37"/>
+      <c r="I35" s="37"/>
+      <c r="J35" s="37"/>
+    </row>
+    <row r="36" spans="1:10" ht="17.850000000000001" customHeight="1">
+      <c r="A36" s="38" t="s">
+        <v>87</v>
+      </c>
+      <c r="B36" s="39"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="39"/>
+      <c r="E36" s="39"/>
+      <c r="F36" s="39"/>
+      <c r="G36" s="39"/>
+      <c r="H36" s="39"/>
+      <c r="I36" s="39"/>
+      <c r="J36" s="40"/>
+    </row>
+    <row r="37" spans="1:10" ht="13.7" customHeight="1">
+      <c r="A37" s="53" t="s">
+        <v>1</v>
+      </c>
+      <c r="B37" s="43" t="s">
+        <v>2</v>
+      </c>
+      <c r="C37" s="30"/>
+      <c r="D37" s="55" t="s">
+        <v>3</v>
+      </c>
+      <c r="E37" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="E28" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="F28" s="8"/>
-      <c r="G28" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="H28" s="8"/>
-      <c r="I28" s="8"/>
-      <c r="J28" s="9" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="5.25" customHeight="1">
-      <c r="A29" s="52"/>
-      <c r="B29" s="52"/>
-      <c r="C29" s="52"/>
-      <c r="D29" s="52"/>
-      <c r="E29" s="52"/>
-      <c r="F29" s="52"/>
-      <c r="G29" s="52"/>
-      <c r="H29" s="52"/>
-      <c r="I29" s="52"/>
-      <c r="J29" s="52"/>
-    </row>
-    <row r="30" spans="1:10" ht="19.7" customHeight="1">
-      <c r="A30" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="B30" s="4">
-        <v>31051</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="D30" s="6">
-        <v>4</v>
-      </c>
-      <c r="E30" s="8"/>
-      <c r="F30" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="G30" s="8"/>
-      <c r="H30" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="I30" s="8"/>
-      <c r="J30" s="9" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="22.35" customHeight="1">
-      <c r="A31" s="47"/>
-      <c r="B31" s="20">
-        <v>31041</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D31" s="6">
-        <v>4</v>
-      </c>
-      <c r="E31" s="8"/>
-      <c r="F31" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="G31" s="8"/>
-      <c r="H31" s="8"/>
-      <c r="I31" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="J31" s="21" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="22.35" customHeight="1">
-      <c r="A32" s="53" t="s">
-        <v>77</v>
-      </c>
-      <c r="B32" s="22">
-        <v>30745</v>
-      </c>
-      <c r="C32" s="19" t="s">
-        <v>78</v>
-      </c>
-      <c r="D32" s="13">
-        <v>6</v>
-      </c>
-      <c r="E32" s="8"/>
-      <c r="F32" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="G32" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="H32" s="8"/>
-      <c r="I32" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="J32" s="23" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="19.7" customHeight="1">
-      <c r="A33" s="53"/>
-      <c r="B33" s="4">
-        <v>31235</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="D33" s="6">
-        <v>4</v>
-      </c>
-      <c r="E33" s="8"/>
-      <c r="F33" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="G33" s="8"/>
-      <c r="H33" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="I33" s="8"/>
-      <c r="J33" s="9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="19.7" customHeight="1">
-      <c r="A34" s="53"/>
-      <c r="B34" s="20">
-        <v>31042</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D34" s="6">
-        <v>4</v>
-      </c>
-      <c r="E34" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="8"/>
-      <c r="I34" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="J34" s="9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A35" s="24"/>
-      <c r="B35" s="54"/>
-      <c r="C35" s="55"/>
-      <c r="D35" s="55"/>
-      <c r="E35" s="55"/>
-      <c r="F35" s="55"/>
-      <c r="G35" s="55"/>
-      <c r="H35" s="55"/>
-      <c r="I35" s="55"/>
-      <c r="J35" s="55"/>
-    </row>
-    <row r="36" spans="1:10" ht="17.850000000000001" customHeight="1">
-      <c r="A36" s="34" t="s">
-        <v>87</v>
-      </c>
-      <c r="B36" s="35"/>
-      <c r="C36" s="35"/>
-      <c r="D36" s="35"/>
-      <c r="E36" s="35"/>
-      <c r="F36" s="35"/>
-      <c r="G36" s="35"/>
-      <c r="H36" s="35"/>
-      <c r="I36" s="35"/>
-      <c r="J36" s="36"/>
-    </row>
-    <row r="37" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A37" s="37" t="s">
-        <v>1</v>
-      </c>
-      <c r="B37" s="39" t="s">
-        <v>2</v>
-      </c>
-      <c r="C37" s="41" t="s">
-        <v>3</v>
-      </c>
-      <c r="D37" s="2"/>
-      <c r="E37" s="43" t="s">
-        <v>4</v>
-      </c>
-      <c r="F37" s="44"/>
-      <c r="G37" s="44"/>
-      <c r="H37" s="44"/>
-      <c r="I37" s="44"/>
-      <c r="J37" s="45"/>
+      <c r="F37" s="48"/>
+      <c r="G37" s="48"/>
+      <c r="H37" s="48"/>
+      <c r="I37" s="48"/>
+      <c r="J37" s="49"/>
     </row>
     <row r="38" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A38" s="38"/>
-      <c r="B38" s="40"/>
-      <c r="C38" s="42"/>
-      <c r="D38" s="2"/>
+      <c r="A38" s="54"/>
+      <c r="B38" s="44"/>
+      <c r="C38" s="31"/>
+      <c r="D38" s="56"/>
       <c r="E38" s="1" t="s">
         <v>5</v>
       </c>
@@ -4247,213 +4186,201 @@
       <c r="I38" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J38" s="3" t="s">
+      <c r="J38" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A39" s="56" t="s">
+      <c r="A39" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="B39" s="4">
+      <c r="B39" s="3">
         <v>30748</v>
       </c>
-      <c r="C39" s="19" t="s">
+      <c r="C39" s="3"/>
+      <c r="D39" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="D39" s="13">
-        <v>6</v>
-      </c>
-      <c r="E39" s="7" t="s">
+      <c r="E39" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F39" s="8"/>
-      <c r="G39" s="7" t="s">
+      <c r="F39" s="6"/>
+      <c r="G39" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="H39" s="8"/>
-      <c r="I39" s="7" t="s">
+      <c r="H39" s="6"/>
+      <c r="I39" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="J39" s="9" t="s">
+      <c r="J39" s="7" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A40" s="57"/>
-      <c r="B40" s="4">
+      <c r="A40" s="33"/>
+      <c r="B40" s="3">
         <v>31045</v>
       </c>
-      <c r="C40" s="12" t="s">
+      <c r="C40" s="3"/>
+      <c r="D40" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="D40" s="13">
-        <v>6</v>
-      </c>
-      <c r="E40" s="7" t="s">
+      <c r="E40" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="F40" s="8"/>
-      <c r="G40" s="7" t="s">
+      <c r="F40" s="6"/>
+      <c r="G40" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="H40" s="8"/>
-      <c r="I40" s="7" t="s">
+      <c r="H40" s="6"/>
+      <c r="I40" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="J40" s="9" t="s">
+      <c r="J40" s="7" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A41" s="57"/>
-      <c r="B41" s="25">
+      <c r="A41" s="33"/>
+      <c r="B41" s="22">
         <v>30746</v>
       </c>
-      <c r="C41" s="19" t="s">
+      <c r="C41" s="22"/>
+      <c r="D41" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="D41" s="13">
-        <v>6</v>
-      </c>
-      <c r="E41" s="7" t="s">
+      <c r="E41" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="F41" s="8"/>
-      <c r="G41" s="7" t="s">
+      <c r="F41" s="6"/>
+      <c r="G41" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="H41" s="8"/>
-      <c r="I41" s="7" t="s">
+      <c r="H41" s="6"/>
+      <c r="I41" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="J41" s="9" t="s">
+      <c r="J41" s="7" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A42" s="57"/>
-      <c r="B42" s="4">
+      <c r="A42" s="33"/>
+      <c r="B42" s="3">
         <v>31030</v>
       </c>
-      <c r="C42" s="12" t="s">
+      <c r="C42" s="3"/>
+      <c r="D42" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="D42" s="13">
+      <c r="E42" s="6"/>
+      <c r="F42" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G42" s="6"/>
+      <c r="H42" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="I42" s="6"/>
+      <c r="J42" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="20.85" customHeight="1">
+      <c r="A43" s="33"/>
+      <c r="B43" s="22">
+        <v>30749</v>
+      </c>
+      <c r="C43" s="22"/>
+      <c r="D43" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="E43" s="6"/>
+      <c r="F43" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="G43" s="6"/>
+      <c r="H43" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="I43" s="6"/>
+      <c r="J43" s="7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="20.85" customHeight="1">
+      <c r="A44" s="57"/>
+      <c r="B44" s="22">
+        <v>30747</v>
+      </c>
+      <c r="C44" s="22"/>
+      <c r="D44" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="E44" s="6"/>
+      <c r="F44" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="G44" s="6"/>
+      <c r="H44" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="I44" s="6"/>
+      <c r="J44" s="7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="16.350000000000001" customHeight="1">
+      <c r="A45" s="58"/>
+      <c r="B45" s="58"/>
+      <c r="C45" s="58"/>
+      <c r="D45" s="58"/>
+      <c r="E45" s="58"/>
+      <c r="F45" s="58"/>
+      <c r="G45" s="58"/>
+      <c r="H45" s="58"/>
+      <c r="I45" s="58"/>
+      <c r="J45" s="58"/>
+    </row>
+    <row r="46" spans="1:10" ht="16.5" customHeight="1">
+      <c r="A46" s="38" t="s">
+        <v>107</v>
+      </c>
+      <c r="B46" s="39"/>
+      <c r="C46" s="39"/>
+      <c r="D46" s="39"/>
+      <c r="E46" s="39"/>
+      <c r="F46" s="39"/>
+      <c r="G46" s="39"/>
+      <c r="H46" s="39"/>
+      <c r="I46" s="39"/>
+      <c r="J46" s="40"/>
+    </row>
+    <row r="47" spans="1:10" ht="13.7" customHeight="1">
+      <c r="A47" s="53" t="s">
+        <v>1</v>
+      </c>
+      <c r="B47" s="43" t="s">
+        <v>2</v>
+      </c>
+      <c r="C47" s="30"/>
+      <c r="D47" s="55" t="s">
+        <v>3</v>
+      </c>
+      <c r="E47" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="E42" s="8"/>
-      <c r="F42" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G42" s="8"/>
-      <c r="H42" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="I42" s="8"/>
-      <c r="J42" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A43" s="57"/>
-      <c r="B43" s="25">
-        <v>30749</v>
-      </c>
-      <c r="C43" s="19" t="s">
-        <v>102</v>
-      </c>
-      <c r="D43" s="13">
-        <v>4</v>
-      </c>
-      <c r="E43" s="8"/>
-      <c r="F43" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="G43" s="8"/>
-      <c r="H43" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="I43" s="8"/>
-      <c r="J43" s="9" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A44" s="58"/>
-      <c r="B44" s="25">
-        <v>30747</v>
-      </c>
-      <c r="C44" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="D44" s="13">
-        <v>4</v>
-      </c>
-      <c r="E44" s="8"/>
-      <c r="F44" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="G44" s="8"/>
-      <c r="H44" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="I44" s="8"/>
-      <c r="J44" s="9" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" ht="16.350000000000001" customHeight="1">
-      <c r="A45" s="59"/>
-      <c r="B45" s="59"/>
-      <c r="C45" s="59"/>
-      <c r="D45" s="59"/>
-      <c r="E45" s="59"/>
-      <c r="F45" s="59"/>
-      <c r="G45" s="59"/>
-      <c r="H45" s="59"/>
-      <c r="I45" s="59"/>
-      <c r="J45" s="59"/>
-    </row>
-    <row r="46" spans="1:10" ht="16.5" customHeight="1">
-      <c r="A46" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="B46" s="35"/>
-      <c r="C46" s="35"/>
-      <c r="D46" s="35"/>
-      <c r="E46" s="35"/>
-      <c r="F46" s="35"/>
-      <c r="G46" s="35"/>
-      <c r="H46" s="35"/>
-      <c r="I46" s="35"/>
-      <c r="J46" s="36"/>
-    </row>
-    <row r="47" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A47" s="37" t="s">
-        <v>1</v>
-      </c>
-      <c r="B47" s="39" t="s">
-        <v>2</v>
-      </c>
-      <c r="C47" s="41" t="s">
-        <v>3</v>
-      </c>
-      <c r="D47" s="2"/>
-      <c r="E47" s="43" t="s">
-        <v>4</v>
-      </c>
-      <c r="F47" s="44"/>
-      <c r="G47" s="44"/>
-      <c r="H47" s="44"/>
-      <c r="I47" s="44"/>
-      <c r="J47" s="45"/>
+      <c r="F47" s="48"/>
+      <c r="G47" s="48"/>
+      <c r="H47" s="48"/>
+      <c r="I47" s="48"/>
+      <c r="J47" s="49"/>
     </row>
     <row r="48" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A48" s="38"/>
-      <c r="B48" s="40"/>
-      <c r="C48" s="42"/>
-      <c r="D48" s="2"/>
+      <c r="A48" s="54"/>
+      <c r="B48" s="44"/>
+      <c r="C48" s="31"/>
+      <c r="D48" s="56"/>
       <c r="E48" s="1" t="s">
         <v>5</v>
       </c>
@@ -4469,197 +4396,185 @@
       <c r="I48" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J48" s="3" t="s">
+      <c r="J48" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A49" s="56" t="s">
+      <c r="A49" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="B49" s="4">
+      <c r="B49" s="3">
         <v>30754</v>
       </c>
-      <c r="C49" s="10" t="s">
+      <c r="C49" s="3"/>
+      <c r="D49" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="D49" s="6">
-        <v>6</v>
-      </c>
-      <c r="E49" s="7" t="s">
+      <c r="E49" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="F49" s="8"/>
-      <c r="G49" s="7" t="s">
+      <c r="F49" s="6"/>
+      <c r="G49" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="H49" s="8"/>
-      <c r="I49" s="7" t="s">
+      <c r="H49" s="6"/>
+      <c r="I49" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="J49" s="9" t="s">
+      <c r="J49" s="7" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A50" s="57"/>
-      <c r="B50" s="4">
+      <c r="A50" s="33"/>
+      <c r="B50" s="3">
         <v>30752</v>
       </c>
-      <c r="C50" s="10" t="s">
+      <c r="C50" s="3"/>
+      <c r="D50" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="D50" s="6">
-        <v>6</v>
-      </c>
-      <c r="E50" s="7" t="s">
+      <c r="E50" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="F50" s="8"/>
-      <c r="G50" s="7" t="s">
+      <c r="F50" s="6"/>
+      <c r="G50" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="H50" s="8"/>
-      <c r="I50" s="7" t="s">
+      <c r="H50" s="6"/>
+      <c r="I50" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="J50" s="9" t="s">
+      <c r="J50" s="7" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A51" s="57"/>
-      <c r="B51" s="4">
+      <c r="A51" s="33"/>
+      <c r="B51" s="3">
         <v>30753</v>
       </c>
-      <c r="C51" s="10" t="s">
+      <c r="C51" s="3"/>
+      <c r="D51" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="D51" s="6">
-        <v>6</v>
-      </c>
-      <c r="E51" s="8"/>
-      <c r="F51" s="7" t="s">
+      <c r="E51" s="6"/>
+      <c r="F51" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="G51" s="7" t="s">
+      <c r="G51" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="H51" s="8"/>
-      <c r="I51" s="7" t="s">
+      <c r="H51" s="6"/>
+      <c r="I51" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="J51" s="9" t="s">
+      <c r="J51" s="7" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A52" s="57"/>
-      <c r="B52" s="4">
+      <c r="A52" s="33"/>
+      <c r="B52" s="3">
         <v>30751</v>
       </c>
-      <c r="C52" s="10" t="s">
+      <c r="C52" s="3"/>
+      <c r="D52" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="D52" s="6">
+      <c r="E52" s="6"/>
+      <c r="F52" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="G52" s="6"/>
+      <c r="H52" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="I52" s="6"/>
+      <c r="J52" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="20.85" customHeight="1">
+      <c r="A53" s="33"/>
+      <c r="B53" s="3">
+        <v>30750</v>
+      </c>
+      <c r="C53" s="3"/>
+      <c r="D53" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="E53" s="6"/>
+      <c r="F53" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="G53" s="6"/>
+      <c r="H53" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="I53" s="6"/>
+      <c r="J53" s="7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="60.6" customHeight="1">
+      <c r="A54" s="57"/>
+      <c r="B54" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="C54" s="23"/>
+      <c r="D54" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="E54" s="50" t="s">
+        <v>124</v>
+      </c>
+      <c r="F54" s="51"/>
+      <c r="G54" s="51"/>
+      <c r="H54" s="51"/>
+      <c r="I54" s="52"/>
+      <c r="J54" s="24"/>
+    </row>
+    <row r="55" spans="1:10" ht="18.95" customHeight="1">
+      <c r="A55" s="38" t="s">
+        <v>125</v>
+      </c>
+      <c r="B55" s="39"/>
+      <c r="C55" s="39"/>
+      <c r="D55" s="39"/>
+      <c r="E55" s="39"/>
+      <c r="F55" s="39"/>
+      <c r="G55" s="39"/>
+      <c r="H55" s="39"/>
+      <c r="I55" s="39"/>
+      <c r="J55" s="40"/>
+    </row>
+    <row r="56" spans="1:10" ht="13.7" customHeight="1">
+      <c r="A56" s="53" t="s">
+        <v>1</v>
+      </c>
+      <c r="B56" s="43" t="s">
+        <v>2</v>
+      </c>
+      <c r="C56" s="30"/>
+      <c r="D56" s="55" t="s">
+        <v>3</v>
+      </c>
+      <c r="E56" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="E52" s="8"/>
-      <c r="F52" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="G52" s="8"/>
-      <c r="H52" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="I52" s="8"/>
-      <c r="J52" s="9" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A53" s="57"/>
-      <c r="B53" s="4">
-        <v>30750</v>
-      </c>
-      <c r="C53" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="D53" s="6">
-        <v>4</v>
-      </c>
-      <c r="E53" s="8"/>
-      <c r="F53" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="G53" s="8"/>
-      <c r="H53" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="I53" s="8"/>
-      <c r="J53" s="9" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="60.6" customHeight="1">
-      <c r="A54" s="58"/>
-      <c r="B54" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="C54" s="19" t="s">
-        <v>123</v>
-      </c>
-      <c r="D54" s="13">
-        <v>4</v>
-      </c>
-      <c r="E54" s="60" t="s">
-        <v>124</v>
-      </c>
-      <c r="F54" s="61"/>
-      <c r="G54" s="61"/>
-      <c r="H54" s="61"/>
-      <c r="I54" s="62"/>
-      <c r="J54" s="27"/>
-    </row>
-    <row r="55" spans="1:10" ht="18.95" customHeight="1">
-      <c r="A55" s="34" t="s">
-        <v>125</v>
-      </c>
-      <c r="B55" s="35"/>
-      <c r="C55" s="35"/>
-      <c r="D55" s="35"/>
-      <c r="E55" s="35"/>
-      <c r="F55" s="35"/>
-      <c r="G55" s="35"/>
-      <c r="H55" s="35"/>
-      <c r="I55" s="35"/>
-      <c r="J55" s="36"/>
-    </row>
-    <row r="56" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A56" s="37" t="s">
-        <v>1</v>
-      </c>
-      <c r="B56" s="39" t="s">
-        <v>2</v>
-      </c>
-      <c r="C56" s="41" t="s">
-        <v>3</v>
-      </c>
-      <c r="D56" s="2"/>
-      <c r="E56" s="43" t="s">
-        <v>4</v>
-      </c>
-      <c r="F56" s="44"/>
-      <c r="G56" s="44"/>
-      <c r="H56" s="44"/>
-      <c r="I56" s="44"/>
-      <c r="J56" s="45"/>
+      <c r="F56" s="48"/>
+      <c r="G56" s="48"/>
+      <c r="H56" s="48"/>
+      <c r="I56" s="48"/>
+      <c r="J56" s="49"/>
     </row>
     <row r="57" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A57" s="38"/>
-      <c r="B57" s="40"/>
-      <c r="C57" s="42"/>
-      <c r="D57" s="2"/>
+      <c r="A57" s="54"/>
+      <c r="B57" s="44"/>
+      <c r="C57" s="31"/>
+      <c r="D57" s="56"/>
       <c r="E57" s="1" t="s">
         <v>5</v>
       </c>
@@ -4675,185 +4590,175 @@
       <c r="I57" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J57" s="3" t="s">
+      <c r="J57" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A58" s="56" t="s">
+      <c r="A58" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="B58" s="4">
+      <c r="B58" s="3">
         <v>30755</v>
       </c>
-      <c r="C58" s="10" t="s">
+      <c r="C58" s="3"/>
+      <c r="D58" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="D58" s="6">
-        <v>6</v>
-      </c>
-      <c r="E58" s="7" t="s">
+      <c r="E58" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="F58" s="8"/>
-      <c r="G58" s="7" t="s">
+      <c r="F58" s="6"/>
+      <c r="G58" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H58" s="8"/>
-      <c r="I58" s="7" t="s">
+      <c r="H58" s="6"/>
+      <c r="I58" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="J58" s="9" t="s">
+      <c r="J58" s="7" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A59" s="57"/>
-      <c r="B59" s="4">
+      <c r="A59" s="33"/>
+      <c r="B59" s="3">
         <v>30757</v>
       </c>
-      <c r="C59" s="10" t="s">
+      <c r="C59" s="3"/>
+      <c r="D59" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="D59" s="6">
-        <v>6</v>
-      </c>
-      <c r="E59" s="7" t="s">
+      <c r="E59" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="F59" s="8"/>
-      <c r="G59" s="7" t="s">
+      <c r="F59" s="6"/>
+      <c r="G59" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="H59" s="8"/>
-      <c r="I59" s="7" t="s">
+      <c r="H59" s="6"/>
+      <c r="I59" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="J59" s="9" t="s">
+      <c r="J59" s="7" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A60" s="57"/>
-      <c r="B60" s="4">
+      <c r="A60" s="33"/>
+      <c r="B60" s="3">
         <v>30758</v>
       </c>
-      <c r="C60" s="10" t="s">
+      <c r="C60" s="3"/>
+      <c r="D60" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="D60" s="6">
-        <v>6</v>
-      </c>
-      <c r="E60" s="8"/>
-      <c r="F60" s="7" t="s">
+      <c r="E60" s="6"/>
+      <c r="F60" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G60" s="8"/>
-      <c r="H60" s="7" t="s">
+      <c r="G60" s="6"/>
+      <c r="H60" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="I60" s="7" t="s">
+      <c r="I60" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="J60" s="9" t="s">
+      <c r="J60" s="7" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A61" s="57"/>
-      <c r="B61" s="4">
+      <c r="A61" s="33"/>
+      <c r="B61" s="3">
         <v>30761</v>
       </c>
-      <c r="C61" s="10" t="s">
+      <c r="C61" s="3"/>
+      <c r="D61" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="D61" s="6">
+      <c r="E61" s="6"/>
+      <c r="F61" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="G61" s="6"/>
+      <c r="H61" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="I61" s="6"/>
+      <c r="J61" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="48.75" customHeight="1">
+      <c r="A62" s="33"/>
+      <c r="B62" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="C62" s="23"/>
+      <c r="D62" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="E62" s="50" t="s">
+        <v>135</v>
+      </c>
+      <c r="F62" s="51"/>
+      <c r="G62" s="51"/>
+      <c r="H62" s="51"/>
+      <c r="I62" s="52"/>
+      <c r="J62" s="24"/>
+    </row>
+    <row r="63" spans="1:10" ht="22.5" customHeight="1">
+      <c r="A63" s="37"/>
+      <c r="B63" s="37"/>
+      <c r="C63" s="37"/>
+      <c r="D63" s="37"/>
+      <c r="E63" s="37"/>
+      <c r="F63" s="37"/>
+      <c r="G63" s="37"/>
+      <c r="H63" s="37"/>
+      <c r="I63" s="37"/>
+      <c r="J63" s="37"/>
+    </row>
+    <row r="64" spans="1:10" ht="18.600000000000001" customHeight="1">
+      <c r="A64" s="38" t="s">
+        <v>136</v>
+      </c>
+      <c r="B64" s="39"/>
+      <c r="C64" s="39"/>
+      <c r="D64" s="39"/>
+      <c r="E64" s="39"/>
+      <c r="F64" s="39"/>
+      <c r="G64" s="39"/>
+      <c r="H64" s="39"/>
+      <c r="I64" s="39"/>
+      <c r="J64" s="40"/>
+    </row>
+    <row r="65" spans="1:10" ht="13.7" customHeight="1">
+      <c r="A65" s="53" t="s">
+        <v>1</v>
+      </c>
+      <c r="B65" s="43" t="s">
+        <v>2</v>
+      </c>
+      <c r="C65" s="30"/>
+      <c r="D65" s="55" t="s">
+        <v>3</v>
+      </c>
+      <c r="E65" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="E61" s="8"/>
-      <c r="F61" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="G61" s="8"/>
-      <c r="H61" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="I61" s="8"/>
-      <c r="J61" s="9" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" ht="48.75" customHeight="1">
-      <c r="A62" s="57"/>
-      <c r="B62" s="26" t="s">
-        <v>133</v>
-      </c>
-      <c r="C62" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="D62" s="13">
-        <v>4</v>
-      </c>
-      <c r="E62" s="60" t="s">
-        <v>135</v>
-      </c>
-      <c r="F62" s="61"/>
-      <c r="G62" s="61"/>
-      <c r="H62" s="61"/>
-      <c r="I62" s="62"/>
-      <c r="J62" s="27"/>
-    </row>
-    <row r="63" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A63" s="55"/>
-      <c r="B63" s="55"/>
-      <c r="C63" s="55"/>
-      <c r="D63" s="55"/>
-      <c r="E63" s="55"/>
-      <c r="F63" s="55"/>
-      <c r="G63" s="55"/>
-      <c r="H63" s="55"/>
-      <c r="I63" s="55"/>
-      <c r="J63" s="55"/>
-    </row>
-    <row r="64" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A64" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="B64" s="35"/>
-      <c r="C64" s="35"/>
-      <c r="D64" s="35"/>
-      <c r="E64" s="35"/>
-      <c r="F64" s="35"/>
-      <c r="G64" s="35"/>
-      <c r="H64" s="35"/>
-      <c r="I64" s="35"/>
-      <c r="J64" s="36"/>
-    </row>
-    <row r="65" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A65" s="37" t="s">
-        <v>1</v>
-      </c>
-      <c r="B65" s="39" t="s">
-        <v>2</v>
-      </c>
-      <c r="C65" s="41" t="s">
-        <v>3</v>
-      </c>
-      <c r="D65" s="2"/>
-      <c r="E65" s="43" t="s">
-        <v>4</v>
-      </c>
-      <c r="F65" s="44"/>
-      <c r="G65" s="44"/>
-      <c r="H65" s="44"/>
-      <c r="I65" s="44"/>
-      <c r="J65" s="45"/>
+      <c r="F65" s="48"/>
+      <c r="G65" s="48"/>
+      <c r="H65" s="48"/>
+      <c r="I65" s="48"/>
+      <c r="J65" s="49"/>
     </row>
     <row r="66" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A66" s="38"/>
-      <c r="B66" s="40"/>
-      <c r="C66" s="42"/>
-      <c r="D66" s="2"/>
+      <c r="A66" s="54"/>
+      <c r="B66" s="44"/>
+      <c r="C66" s="31"/>
+      <c r="D66" s="56"/>
       <c r="E66" s="1" t="s">
         <v>5</v>
       </c>
@@ -4869,187 +4774,177 @@
       <c r="I66" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J66" s="3" t="s">
+      <c r="J66" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="67" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A67" s="56" t="s">
+      <c r="A67" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="B67" s="4">
+      <c r="B67" s="3">
         <v>30768</v>
       </c>
-      <c r="C67" s="10" t="s">
+      <c r="C67" s="3"/>
+      <c r="D67" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="D67" s="6">
-        <v>6</v>
-      </c>
-      <c r="E67" s="7" t="s">
+      <c r="E67" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="F67" s="8"/>
-      <c r="G67" s="7" t="s">
+      <c r="F67" s="6"/>
+      <c r="G67" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="H67" s="8"/>
-      <c r="I67" s="7" t="s">
+      <c r="H67" s="6"/>
+      <c r="I67" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="J67" s="9" t="s">
+      <c r="J67" s="7" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="68" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A68" s="57"/>
-      <c r="B68" s="4">
+      <c r="A68" s="33"/>
+      <c r="B68" s="3">
         <v>30763</v>
       </c>
-      <c r="C68" s="10" t="s">
+      <c r="C68" s="3"/>
+      <c r="D68" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="D68" s="6">
-        <v>6</v>
-      </c>
-      <c r="E68" s="7" t="s">
+      <c r="E68" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="F68" s="8"/>
-      <c r="G68" s="7" t="s">
+      <c r="F68" s="6"/>
+      <c r="G68" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="H68" s="8"/>
-      <c r="I68" s="7" t="s">
+      <c r="H68" s="6"/>
+      <c r="I68" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="J68" s="9" t="s">
+      <c r="J68" s="7" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="69" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A69" s="57"/>
-      <c r="B69" s="4">
+      <c r="A69" s="33"/>
+      <c r="B69" s="3">
         <v>30774</v>
       </c>
-      <c r="C69" s="10" t="s">
+      <c r="C69" s="3"/>
+      <c r="D69" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="D69" s="6">
+      <c r="E69" s="6"/>
+      <c r="F69" s="6"/>
+      <c r="G69" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="H69" s="6"/>
+      <c r="I69" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="J69" s="7" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ht="20.85" customHeight="1">
+      <c r="A70" s="33"/>
+      <c r="B70" s="3">
+        <v>30765</v>
+      </c>
+      <c r="C70" s="3"/>
+      <c r="D70" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="E70" s="6"/>
+      <c r="F70" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="G70" s="6"/>
+      <c r="H70" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I70" s="6"/>
+      <c r="J70" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" ht="20.85" customHeight="1">
+      <c r="A71" s="33"/>
+      <c r="B71" s="13">
+        <v>30775</v>
+      </c>
+      <c r="C71" s="13"/>
+      <c r="D71" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E71" s="6"/>
+      <c r="F71" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="G71" s="6"/>
+      <c r="H71" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="I71" s="6"/>
+      <c r="J71" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" ht="23.25" customHeight="1">
+      <c r="A72" s="37"/>
+      <c r="B72" s="37"/>
+      <c r="C72" s="37"/>
+      <c r="D72" s="37"/>
+      <c r="E72" s="37"/>
+      <c r="F72" s="37"/>
+      <c r="G72" s="37"/>
+      <c r="H72" s="37"/>
+      <c r="I72" s="37"/>
+      <c r="J72" s="37"/>
+    </row>
+    <row r="73" spans="1:10" ht="18.95" customHeight="1">
+      <c r="A73" s="38" t="s">
+        <v>145</v>
+      </c>
+      <c r="B73" s="39"/>
+      <c r="C73" s="39"/>
+      <c r="D73" s="39"/>
+      <c r="E73" s="39"/>
+      <c r="F73" s="39"/>
+      <c r="G73" s="39"/>
+      <c r="H73" s="39"/>
+      <c r="I73" s="39"/>
+      <c r="J73" s="40"/>
+    </row>
+    <row r="74" spans="1:10" ht="12.6" customHeight="1">
+      <c r="A74" s="41" t="s">
+        <v>1</v>
+      </c>
+      <c r="B74" s="43" t="s">
+        <v>2</v>
+      </c>
+      <c r="C74" s="30"/>
+      <c r="D74" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="E74" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="E69" s="8"/>
-      <c r="F69" s="8"/>
-      <c r="G69" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="H69" s="8"/>
-      <c r="I69" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="J69" s="9" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A70" s="57"/>
-      <c r="B70" s="4">
-        <v>30765</v>
-      </c>
-      <c r="C70" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="D70" s="6">
-        <v>4</v>
-      </c>
-      <c r="E70" s="8"/>
-      <c r="F70" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="G70" s="8"/>
-      <c r="H70" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="I70" s="8"/>
-      <c r="J70" s="9" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A71" s="57"/>
-      <c r="B71" s="16">
-        <v>30775</v>
-      </c>
-      <c r="C71" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="D71" s="6">
-        <v>4</v>
-      </c>
-      <c r="E71" s="8"/>
-      <c r="F71" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="G71" s="8"/>
-      <c r="H71" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="I71" s="8"/>
-      <c r="J71" s="9" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" ht="23.25" customHeight="1">
-      <c r="A72" s="55"/>
-      <c r="B72" s="55"/>
-      <c r="C72" s="55"/>
-      <c r="D72" s="55"/>
-      <c r="E72" s="55"/>
-      <c r="F72" s="55"/>
-      <c r="G72" s="55"/>
-      <c r="H72" s="55"/>
-      <c r="I72" s="55"/>
-      <c r="J72" s="55"/>
-    </row>
-    <row r="73" spans="1:10" ht="18.95" customHeight="1">
-      <c r="A73" s="34" t="s">
-        <v>145</v>
-      </c>
-      <c r="B73" s="35"/>
-      <c r="C73" s="35"/>
-      <c r="D73" s="35"/>
-      <c r="E73" s="35"/>
-      <c r="F73" s="35"/>
-      <c r="G73" s="35"/>
-      <c r="H73" s="35"/>
-      <c r="I73" s="35"/>
-      <c r="J73" s="36"/>
-    </row>
-    <row r="74" spans="1:10" ht="12.6" customHeight="1">
-      <c r="A74" s="63" t="s">
-        <v>1</v>
-      </c>
-      <c r="B74" s="39" t="s">
-        <v>2</v>
-      </c>
-      <c r="C74" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="D74" s="28"/>
-      <c r="E74" s="43" t="s">
-        <v>4</v>
-      </c>
-      <c r="F74" s="44"/>
-      <c r="G74" s="44"/>
-      <c r="H74" s="44"/>
-      <c r="I74" s="44"/>
-      <c r="J74" s="45"/>
+      <c r="F74" s="48"/>
+      <c r="G74" s="48"/>
+      <c r="H74" s="48"/>
+      <c r="I74" s="48"/>
+      <c r="J74" s="49"/>
     </row>
     <row r="75" spans="1:10" ht="12.6" customHeight="1">
-      <c r="A75" s="64"/>
-      <c r="B75" s="40"/>
-      <c r="C75" s="66"/>
-      <c r="D75" s="28"/>
+      <c r="A75" s="42"/>
+      <c r="B75" s="44"/>
+      <c r="C75" s="31"/>
+      <c r="D75" s="46"/>
       <c r="E75" s="1" t="s">
         <v>5</v>
       </c>
@@ -5065,140 +4960,328 @@
       <c r="I75" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J75" s="3" t="s">
+      <c r="J75" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="76" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A76" s="56" t="s">
+      <c r="A76" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="B76" s="4">
+      <c r="B76" s="3">
         <v>30776</v>
       </c>
-      <c r="C76" s="10" t="s">
+      <c r="C76" s="3"/>
+      <c r="D76" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="D76" s="6">
+      <c r="E76" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="F76" s="6"/>
+      <c r="G76" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="H76" s="6"/>
+      <c r="I76" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="J76" s="7" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" ht="20.85" customHeight="1">
+      <c r="A77" s="33"/>
+      <c r="B77" s="3">
+        <v>30792</v>
+      </c>
+      <c r="C77" s="3"/>
+      <c r="D77" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="E77" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="F77" s="6"/>
+      <c r="G77" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="H77" s="6"/>
+      <c r="I77" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="J77" s="7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" ht="20.85" customHeight="1">
+      <c r="A78" s="33"/>
+      <c r="B78" s="3">
+        <v>30786</v>
+      </c>
+      <c r="C78" s="3"/>
+      <c r="D78" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="E78" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="F78" s="6"/>
+      <c r="G78" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="H78" s="6"/>
+      <c r="I78" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="J78" s="7" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" ht="20.85" customHeight="1">
+      <c r="A79" s="33"/>
+      <c r="B79" s="3">
+        <v>30789</v>
+      </c>
+      <c r="C79" s="3"/>
+      <c r="D79" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="E79" s="6"/>
+      <c r="F79" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="G79" s="6"/>
+      <c r="H79" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="I79" s="6"/>
+      <c r="J79" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" ht="20.85" customHeight="1">
+      <c r="A80" s="33"/>
+      <c r="B80" s="3">
+        <v>30783</v>
+      </c>
+      <c r="C80" s="3"/>
+      <c r="D80" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="E80" s="6"/>
+      <c r="F80" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="G80" s="6"/>
+      <c r="H80" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="I80" s="6"/>
+      <c r="J80" s="7" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" ht="15">
+      <c r="A82" s="73" t="s">
+        <v>181</v>
+      </c>
+      <c r="B82" s="39"/>
+      <c r="C82" s="39"/>
+      <c r="D82" s="39"/>
+      <c r="E82" s="39"/>
+      <c r="F82" s="39"/>
+      <c r="G82" s="39"/>
+      <c r="H82" s="39"/>
+      <c r="I82" s="39"/>
+      <c r="J82" s="40"/>
+    </row>
+    <row r="83" spans="1:10">
+      <c r="A83" s="41" t="s">
+        <v>1</v>
+      </c>
+      <c r="B83" s="43" t="s">
+        <v>2</v>
+      </c>
+      <c r="C83" s="30"/>
+      <c r="D83" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="E83" s="47" t="s">
+        <v>4</v>
+      </c>
+      <c r="F83" s="48"/>
+      <c r="G83" s="48"/>
+      <c r="H83" s="48"/>
+      <c r="I83" s="48"/>
+      <c r="J83" s="49"/>
+    </row>
+    <row r="84" spans="1:10">
+      <c r="A84" s="42"/>
+      <c r="B84" s="44"/>
+      <c r="C84" s="31"/>
+      <c r="D84" s="46"/>
+      <c r="E84" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F84" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E76" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="F76" s="8"/>
-      <c r="G76" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="H76" s="8"/>
-      <c r="I76" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="J76" s="9" t="s">
+      <c r="G84" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I84" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J84" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" ht="18">
+      <c r="A85" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B85" s="3">
+        <v>30795</v>
+      </c>
+      <c r="C85" s="3"/>
+      <c r="D85" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="E85" s="6"/>
+      <c r="F85" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="G85" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="H85" s="6"/>
+      <c r="I85" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="J85" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" ht="27">
+      <c r="A86" s="33"/>
+      <c r="B86" s="3">
+        <v>30798</v>
+      </c>
+      <c r="C86" s="3"/>
+      <c r="D86" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="E86" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="F86" s="6"/>
+      <c r="G86" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="H86" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="I86" s="6"/>
+      <c r="J86" s="7" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A77" s="57"/>
-      <c r="B77" s="4">
-        <v>30792</v>
-      </c>
-      <c r="C77" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="D77" s="6">
-        <v>6</v>
-      </c>
-      <c r="E77" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="F77" s="8"/>
-      <c r="G77" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="H77" s="8"/>
-      <c r="I77" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="J77" s="9" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A78" s="57"/>
-      <c r="B78" s="4">
-        <v>30786</v>
-      </c>
-      <c r="C78" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="D78" s="6">
-        <v>6</v>
-      </c>
-      <c r="E78" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="F78" s="8"/>
-      <c r="G78" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="H78" s="8"/>
-      <c r="I78" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="J78" s="9" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A79" s="57"/>
-      <c r="B79" s="4">
-        <v>30789</v>
-      </c>
-      <c r="C79" s="10" t="s">
-        <v>153</v>
-      </c>
-      <c r="D79" s="6">
-        <v>4</v>
-      </c>
-      <c r="E79" s="8"/>
-      <c r="F79" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="G79" s="8"/>
-      <c r="H79" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="I79" s="8"/>
-      <c r="J79" s="9" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A80" s="57"/>
-      <c r="B80" s="4">
-        <v>30783</v>
-      </c>
-      <c r="C80" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="D80" s="6">
-        <v>4</v>
-      </c>
-      <c r="E80" s="8"/>
-      <c r="F80" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="G80" s="8"/>
-      <c r="H80" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="I80" s="8"/>
-      <c r="J80" s="9" t="s">
-        <v>157</v>
+    <row r="87" spans="1:10" ht="27">
+      <c r="A87" s="33"/>
+      <c r="B87" s="3">
+        <v>30800</v>
+      </c>
+      <c r="C87" s="3"/>
+      <c r="D87" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="E87" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="F87" s="6"/>
+      <c r="G87" s="6"/>
+      <c r="H87" s="6"/>
+      <c r="I87" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="J87" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" ht="27">
+      <c r="A88" s="57"/>
+      <c r="B88" s="3">
+        <v>31272</v>
+      </c>
+      <c r="C88" s="3"/>
+      <c r="D88" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="E88" s="6"/>
+      <c r="F88" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="G88" s="6"/>
+      <c r="H88" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="I88" s="6"/>
+      <c r="J88" s="7" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="57">
+  <mergeCells count="62">
+    <mergeCell ref="A85:A88"/>
+    <mergeCell ref="A82:J82"/>
+    <mergeCell ref="A83:A84"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="D83:D84"/>
+    <mergeCell ref="E83:J83"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="A7:A13"/>
+    <mergeCell ref="A15:A21"/>
+    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="A23:J23"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:J24"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="B35:J35"/>
+    <mergeCell ref="A36:J36"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="E37:J37"/>
+    <mergeCell ref="A39:A44"/>
+    <mergeCell ref="A45:J45"/>
+    <mergeCell ref="A46:J46"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="D47:D48"/>
+    <mergeCell ref="E47:J47"/>
+    <mergeCell ref="D65:D66"/>
+    <mergeCell ref="E65:J65"/>
+    <mergeCell ref="A49:A54"/>
+    <mergeCell ref="E54:I54"/>
+    <mergeCell ref="A55:J55"/>
+    <mergeCell ref="A56:A57"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="E56:J56"/>
     <mergeCell ref="A76:A80"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
@@ -5207,7 +5290,7 @@
     <mergeCell ref="A73:J73"/>
     <mergeCell ref="A74:A75"/>
     <mergeCell ref="B74:B75"/>
-    <mergeCell ref="C74:C75"/>
+    <mergeCell ref="D74:D75"/>
     <mergeCell ref="E74:J74"/>
     <mergeCell ref="A58:A62"/>
     <mergeCell ref="E62:I62"/>
@@ -5215,47 +5298,6 @@
     <mergeCell ref="A64:J64"/>
     <mergeCell ref="A65:A66"/>
     <mergeCell ref="B65:B66"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="E65:J65"/>
-    <mergeCell ref="A49:A54"/>
-    <mergeCell ref="E54:I54"/>
-    <mergeCell ref="A55:J55"/>
-    <mergeCell ref="A56:A57"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="C56:C57"/>
-    <mergeCell ref="E56:J56"/>
-    <mergeCell ref="A45:J45"/>
-    <mergeCell ref="A46:J46"/>
-    <mergeCell ref="A47:A48"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="E47:J47"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="E37:J37"/>
-    <mergeCell ref="A39:A44"/>
-    <mergeCell ref="A29:J29"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="A32:A34"/>
-    <mergeCell ref="B35:J35"/>
-    <mergeCell ref="A36:J36"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="E24:J24"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="A7:A13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="A15:A21"/>
-    <mergeCell ref="A22:J22"/>
-    <mergeCell ref="A23:J23"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="E5:J5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5279,241 +5321,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21.75" customHeight="1">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="68" t="s">
         <v>179</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74"/>
-      <c r="F1" s="74"/>
-      <c r="G1" s="74"/>
-      <c r="H1" s="74"/>
-      <c r="I1" s="74"/>
-      <c r="J1" s="74"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
     </row>
     <row r="2" spans="1:10" ht="15.75">
-      <c r="A2" s="75" t="s">
+      <c r="A2" s="70" t="s">
         <v>180</v>
       </c>
-      <c r="B2" s="75"/>
-      <c r="C2" s="75"/>
-      <c r="D2" s="75"/>
-      <c r="E2" s="75"/>
-      <c r="F2" s="75"/>
-      <c r="G2" s="75"/>
-      <c r="H2" s="75"/>
-      <c r="I2" s="75"/>
-      <c r="J2" s="75"/>
-    </row>
-    <row r="3" spans="1:10" ht="24.75" customHeight="1">
-      <c r="A3" s="69" t="s">
-        <v>181</v>
-      </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="35"/>
-      <c r="G3" s="35"/>
-      <c r="H3" s="35"/>
-      <c r="I3" s="35"/>
-      <c r="J3" s="36"/>
-    </row>
-    <row r="4" spans="1:10" ht="12.6" customHeight="1">
-      <c r="A4" s="63" t="s">
+      <c r="B2" s="70"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="70"/>
+      <c r="E2" s="70"/>
+      <c r="F2" s="70"/>
+      <c r="G2" s="70"/>
+      <c r="H2" s="70"/>
+      <c r="I2" s="70"/>
+      <c r="J2" s="70"/>
+    </row>
+    <row r="3" spans="1:10" ht="24.75" customHeight="1"/>
+    <row r="4" spans="1:10" ht="12.6" customHeight="1"/>
+    <row r="5" spans="1:10" ht="12.6" customHeight="1"/>
+    <row r="6" spans="1:10" ht="20.85" customHeight="1"/>
+    <row r="7" spans="1:10" ht="20.85" customHeight="1"/>
+    <row r="8" spans="1:10" ht="20.85" customHeight="1"/>
+    <row r="9" spans="1:10" ht="20.85" customHeight="1"/>
+    <row r="10" spans="1:10" ht="14.25" customHeight="1">
+      <c r="A10" s="58"/>
+      <c r="B10" s="58"/>
+      <c r="C10" s="58"/>
+      <c r="D10" s="58"/>
+      <c r="E10" s="58"/>
+      <c r="F10" s="58"/>
+      <c r="G10" s="58"/>
+      <c r="H10" s="58"/>
+      <c r="I10" s="58"/>
+      <c r="J10" s="58"/>
+    </row>
+    <row r="11" spans="1:10" ht="20.85" customHeight="1">
+      <c r="A11" s="38" t="s">
+        <v>167</v>
+      </c>
+      <c r="B11" s="39"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="39"/>
+      <c r="I11" s="39"/>
+      <c r="J11" s="40"/>
+    </row>
+    <row r="12" spans="1:10" ht="12.6" customHeight="1">
+      <c r="A12" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="39" t="s">
+      <c r="B12" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="28"/>
-      <c r="E4" s="43" t="s">
+      <c r="C12" s="71"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="44"/>
-      <c r="G4" s="44"/>
-      <c r="H4" s="44"/>
-      <c r="I4" s="44"/>
-      <c r="J4" s="45"/>
-    </row>
-    <row r="5" spans="1:10" ht="12.6" customHeight="1">
-      <c r="A5" s="64"/>
-      <c r="B5" s="40"/>
-      <c r="C5" s="66"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A6" s="56" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="4">
-        <v>30795</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="D6" s="6">
-        <v>6</v>
-      </c>
-      <c r="E6" s="8"/>
-      <c r="F6" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="H6" s="8"/>
-      <c r="I6" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="J6" s="9" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A7" s="57"/>
-      <c r="B7" s="4">
-        <v>30798</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="D7" s="6">
-        <v>6</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="I7" s="8"/>
-      <c r="J7" s="9" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A8" s="57"/>
-      <c r="B8" s="4">
-        <v>30800</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="D8" s="6">
-        <v>4</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="J8" s="9" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A9" s="58"/>
-      <c r="B9" s="4">
-        <v>31272</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="D9" s="6">
-        <v>4</v>
-      </c>
-      <c r="E9" s="8"/>
-      <c r="F9" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="G9" s="8"/>
-      <c r="H9" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="I9" s="8"/>
-      <c r="J9" s="9" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A10" s="59"/>
-      <c r="B10" s="59"/>
-      <c r="C10" s="59"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="59"/>
-      <c r="F10" s="59"/>
-      <c r="G10" s="59"/>
-      <c r="H10" s="59"/>
-      <c r="I10" s="59"/>
-      <c r="J10" s="59"/>
-    </row>
-    <row r="11" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A11" s="34" t="s">
-        <v>167</v>
-      </c>
-      <c r="B11" s="35"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="35"/>
-      <c r="J11" s="36"/>
-    </row>
-    <row r="12" spans="1:10" ht="12.6" customHeight="1">
-      <c r="A12" s="63" t="s">
-        <v>1</v>
-      </c>
-      <c r="B12" s="39" t="s">
-        <v>2</v>
-      </c>
-      <c r="C12" s="67"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="43" t="s">
-        <v>4</v>
-      </c>
-      <c r="F12" s="44"/>
-      <c r="G12" s="44"/>
-      <c r="H12" s="44"/>
-      <c r="I12" s="44"/>
-      <c r="J12" s="45"/>
+      <c r="F12" s="48"/>
+      <c r="G12" s="48"/>
+      <c r="H12" s="48"/>
+      <c r="I12" s="48"/>
+      <c r="J12" s="49"/>
     </row>
     <row r="13" spans="1:10" ht="12.6" customHeight="1">
-      <c r="A13" s="64"/>
-      <c r="B13" s="40"/>
-      <c r="C13" s="68"/>
+      <c r="A13" s="42"/>
+      <c r="B13" s="44"/>
+      <c r="C13" s="72"/>
       <c r="D13" s="1" t="s">
         <v>168</v>
       </c>
@@ -5532,287 +5421,281 @@
       <c r="I13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J13" s="3" t="s">
+      <c r="J13" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="12.2" customHeight="1">
-      <c r="A14" s="56" t="s">
+      <c r="A14" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="13">
         <v>30809</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="D14" s="29">
+      <c r="D14" s="26">
         <v>24</v>
       </c>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="9" t="s">
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="7" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="12.2" customHeight="1">
-      <c r="A15" s="57"/>
-      <c r="B15" s="30">
+      <c r="A15" s="33"/>
+      <c r="B15" s="27">
         <v>32404</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="D15" s="29">
+      <c r="D15" s="26">
         <v>2</v>
       </c>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="9" t="s">
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="7" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="12.2" customHeight="1">
-      <c r="A16" s="57"/>
-      <c r="B16" s="30">
+      <c r="A16" s="33"/>
+      <c r="B16" s="27">
         <v>32405</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="D16" s="29">
+      <c r="D16" s="26">
         <v>1</v>
       </c>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="9" t="s">
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="7" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="12.2" customHeight="1">
-      <c r="A17" s="57"/>
-      <c r="B17" s="31">
+      <c r="A17" s="33"/>
+      <c r="B17" s="28">
         <v>32406</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="D17" s="29">
+      <c r="D17" s="26">
         <v>3</v>
       </c>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="9" t="s">
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
+      <c r="I17" s="15"/>
+      <c r="J17" s="7" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="12.2" customHeight="1">
-      <c r="A18" s="57"/>
-      <c r="B18" s="30">
+      <c r="A18" s="33"/>
+      <c r="B18" s="27">
         <v>32407</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="D18" s="29">
+      <c r="D18" s="26">
         <v>2</v>
       </c>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="9" t="s">
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="7" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="12.2" customHeight="1">
-      <c r="A19" s="57"/>
-      <c r="B19" s="31">
+      <c r="A19" s="33"/>
+      <c r="B19" s="28">
         <v>32408</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="D19" s="29">
+      <c r="D19" s="26">
         <v>2</v>
       </c>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="9" t="s">
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="7" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="12.2" customHeight="1">
-      <c r="A20" s="57"/>
-      <c r="B20" s="31">
+      <c r="A20" s="33"/>
+      <c r="B20" s="28">
         <v>32409</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="D20" s="29">
+      <c r="D20" s="26">
         <v>1</v>
       </c>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="9" t="s">
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="7" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="12.2" customHeight="1">
-      <c r="A21" s="57"/>
-      <c r="B21" s="31">
+      <c r="A21" s="33"/>
+      <c r="B21" s="28">
         <v>32410</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="D21" s="29">
+      <c r="D21" s="26">
         <v>5</v>
       </c>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="9" t="s">
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="15"/>
+      <c r="J21" s="7" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="12.2" customHeight="1">
-      <c r="A22" s="57"/>
-      <c r="B22" s="31">
+      <c r="A22" s="33"/>
+      <c r="B22" s="28">
         <v>32411</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="D22" s="29">
+      <c r="D22" s="26">
         <v>5</v>
       </c>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="9" t="s">
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="7" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="12.2" customHeight="1">
-      <c r="A23" s="57"/>
-      <c r="B23" s="31">
+      <c r="A23" s="33"/>
+      <c r="B23" s="28">
         <v>32412</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="D23" s="29">
+      <c r="D23" s="26">
         <v>2</v>
       </c>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="9" t="s">
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="15"/>
+      <c r="I23" s="15"/>
+      <c r="J23" s="7" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="12.2" customHeight="1">
-      <c r="A24" s="57"/>
-      <c r="B24" s="31">
+      <c r="A24" s="33"/>
+      <c r="B24" s="28">
         <v>32413</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="D24" s="29">
+      <c r="D24" s="26">
         <v>1</v>
       </c>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="9" t="s">
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="7" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="12.2" customHeight="1">
-      <c r="A25" s="57"/>
-      <c r="B25" s="30">
+      <c r="A25" s="33"/>
+      <c r="B25" s="27">
         <v>32414</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="D25" s="29">
+      <c r="D25" s="26">
         <v>24</v>
       </c>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
-      <c r="J25" s="9" t="s">
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="7" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A26" s="58"/>
-      <c r="B26" s="16">
+      <c r="A26" s="57"/>
+      <c r="B26" s="13">
         <v>32345</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="D26" s="29">
+      <c r="D26" s="26">
         <v>23</v>
       </c>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="32"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="29"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="9">
     <mergeCell ref="A14:A26"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A6:A9"/>
     <mergeCell ref="A10:J10"/>
     <mergeCell ref="A11:J11"/>
     <mergeCell ref="A12:A13"/>
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="C12:C13"/>
     <mergeCell ref="E12:J12"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="E4:J4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: centralize the relationships in an index
</commit_message>
<xml_diff>
--- a/database/horarios/HORARIO_ITIJ_202551.xlsx
+++ b/database/horarios/HORARIO_ITIJ_202551.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johng\ESPE\Aplicaciones distribuidas\Proyecto\api-shedsync\database\horarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF9040F-469A-4DE5-89C2-E0842411D197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BA0AF3-A195-4917-AF4A-387B921F3C9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="183">
   <si>
     <r>
       <rPr>
@@ -2110,318 +2110,307 @@
     <r>
       <rPr>
         <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>PROGRAMACIÓN AVANZADA</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="6.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">07:00 - 09:00
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Lab DCCO 05</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>ORTIZ DELGADO LUIS ARMANDO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>APLICACIONES DISTRIBUIDAS</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="6.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">11:00 - 13:00
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Lab DCCO 06</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>SEGURIDAD INFORMÁTICA</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="6.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">09:00 - 11:00
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Lab DCCO 01</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>DISEÑO Y EVALUACIÓN DE PROYECTOS TI</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="6.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">09:00 - 11:00
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Lab DCCO 05</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>CEVALLOS FARIAS JAVIER JOSÉ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>MINERIA DE DATOS</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>BENAVIDES ASTUDILLO DIEGO EDUARDO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>GESTIÓN DE LA SEGURIDAD INFORMÁTICA</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="6.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">11:00 - 13:00
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Lab DCCO 03</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="6.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">09:00 - 11:00
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Lab DCCO 02</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>ARQUITECTURA DE SOFTWARE</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>TECNOLOGÍAS EMERGENTES</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="6.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">13:00 - 15:00
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Lab DCCO 04</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>GESTIÓN Y EMPRENDIMIENTO (CADM-A0G00)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">15:00 17:00
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>CD-EN LINEA</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>ARTEAGA MEDINA SANTIAGO ISRAEL</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
         <sz val="11.5"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>SÉPTIMO PERIODO ACADÉMICO ORDINARIO (PAO 7)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>PROGRAMACIÓN AVANZADA</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="6.5"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">07:00 - 09:00
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6.5"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>Lab DCCO 05</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>ORTIZ DELGADO LUIS ARMANDO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>APLICACIONES DISTRIBUIDAS</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="6.5"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">11:00 - 13:00
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6.5"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>Lab DCCO 06</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>SEGURIDAD INFORMÁTICA</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="6.5"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">09:00 - 11:00
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6.5"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>Lab DCCO 01</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>DISEÑO Y EVALUACIÓN DE PROYECTOS TI</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="6.5"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">09:00 - 11:00
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6.5"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>Lab DCCO 05</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>CEVALLOS FARIAS JAVIER JOSÉ</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>MINERIA DE DATOS</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>BENAVIDES ASTUDILLO DIEGO EDUARDO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>GESTIÓN DE LA SEGURIDAD INFORMÁTICA</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="6.5"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">11:00 - 13:00
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6.5"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>Lab DCCO 03</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="6.5"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">09:00 - 11:00
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6.5"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>Lab DCCO 02</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>ARQUITECTURA DE SOFTWARE</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>TECNOLOGÍAS EMERGENTES</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="6.5"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">13:00 - 15:00
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6.5"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>Lab DCCO 04</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>GESTIÓN Y EMPRENDIMIENTO (CADM-A0G00)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">15:00 17:00
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>CD-EN LINEA</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>ARTEAGA MEDINA SANTIAGO ISRAEL</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
       <t>UNIDAD DE INTEGRACIÓN CURRICULAR</t>
     </r>
   </si>
@@ -2554,6 +2543,12 @@
   </si>
   <si>
     <t>HORARIOS DEL PERÍODO ACADÉMICO 202551 - PREGRADO OCTUBRE 2025 - MARZO 2026</t>
+  </si>
+  <si>
+    <t>SÉPTIMO PERIODO ACADÉMICO ORDINARIO (PAO 7)</t>
+  </si>
+  <si>
+    <t>OCTAVO PERIODO ACADÉMICO ORDINARIO (PAO 8)</t>
   </si>
 </sst>
 </file>
@@ -2885,7 +2880,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -2988,6 +2983,102 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2997,99 +3088,6 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -3105,7 +3103,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3427,86 +3425,86 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21.75" customHeight="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="66" t="s">
+        <v>178</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75">
+      <c r="A2" s="68" t="s">
         <v>179</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-    </row>
-    <row r="2" spans="1:10" ht="15.75">
-      <c r="A2" s="36" t="s">
+      <c r="B2" s="68"/>
+      <c r="C2" s="68"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="68"/>
+    </row>
+    <row r="3" spans="1:10" ht="24.75" customHeight="1">
+      <c r="A3" s="47" t="s">
         <v>180</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-    </row>
-    <row r="3" spans="1:10" ht="24.75" customHeight="1">
-      <c r="A3" s="66" t="s">
-        <v>181</v>
-      </c>
-      <c r="B3" s="67"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
     </row>
     <row r="4" spans="1:10" ht="25.7" customHeight="1">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="39"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
-      <c r="I4" s="39"/>
-      <c r="J4" s="40"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="37"/>
     </row>
     <row r="5" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A5" s="53" t="s">
+      <c r="A5" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="40" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="30"/>
-      <c r="D5" s="55" t="s">
+      <c r="D5" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="47" t="s">
+      <c r="E5" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="48"/>
-      <c r="G5" s="48"/>
-      <c r="H5" s="48"/>
-      <c r="I5" s="48"/>
-      <c r="J5" s="49"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="45"/>
+      <c r="I5" s="45"/>
+      <c r="J5" s="46"/>
     </row>
     <row r="6" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A6" s="54"/>
-      <c r="B6" s="44"/>
+      <c r="A6" s="51"/>
+      <c r="B6" s="41"/>
       <c r="C6" s="31"/>
-      <c r="D6" s="56"/>
+      <c r="D6" s="53"/>
       <c r="E6" s="1" t="s">
         <v>5</v>
       </c>
@@ -3527,7 +3525,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A7" s="63" t="s">
+      <c r="A7" s="54" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="3">
@@ -3551,7 +3549,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A8" s="60"/>
+      <c r="A8" s="55"/>
       <c r="B8" s="3">
         <v>29767</v>
       </c>
@@ -3575,7 +3573,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A9" s="60"/>
+      <c r="A9" s="55"/>
       <c r="B9" s="3">
         <v>31036</v>
       </c>
@@ -3599,7 +3597,7 @@
       </c>
     </row>
     <row r="10" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A10" s="60"/>
+      <c r="A10" s="55"/>
       <c r="B10" s="3">
         <v>30530</v>
       </c>
@@ -3619,7 +3617,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="24.2" customHeight="1">
-      <c r="A11" s="60"/>
+      <c r="A11" s="55"/>
       <c r="B11" s="3">
         <v>30534</v>
       </c>
@@ -3639,7 +3637,7 @@
       </c>
     </row>
     <row r="12" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A12" s="60"/>
+      <c r="A12" s="55"/>
       <c r="B12" s="3">
         <v>31545</v>
       </c>
@@ -3661,7 +3659,7 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A13" s="64"/>
+      <c r="A13" s="56"/>
       <c r="B13" s="13">
         <v>28841</v>
       </c>
@@ -3695,7 +3693,7 @@
       <c r="J14" s="15"/>
     </row>
     <row r="15" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A15" s="63" t="s">
+      <c r="A15" s="54" t="s">
         <v>35</v>
       </c>
       <c r="B15" s="3">
@@ -3719,7 +3717,7 @@
       </c>
     </row>
     <row r="16" spans="1:10" ht="23.25" customHeight="1">
-      <c r="A16" s="60"/>
+      <c r="A16" s="55"/>
       <c r="B16" s="3">
         <v>30742</v>
       </c>
@@ -3743,7 +3741,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A17" s="60"/>
+      <c r="A17" s="55"/>
       <c r="B17" s="3">
         <v>31037</v>
       </c>
@@ -3767,7 +3765,7 @@
       </c>
     </row>
     <row r="18" spans="1:10" ht="24.2" customHeight="1">
-      <c r="A18" s="60"/>
+      <c r="A18" s="55"/>
       <c r="B18" s="3">
         <v>31914</v>
       </c>
@@ -3787,7 +3785,7 @@
       </c>
     </row>
     <row r="19" spans="1:10" ht="24.2" customHeight="1">
-      <c r="A19" s="60"/>
+      <c r="A19" s="55"/>
       <c r="B19" s="3">
         <v>30531</v>
       </c>
@@ -3807,7 +3805,7 @@
       </c>
     </row>
     <row r="20" spans="1:10" ht="21.6" customHeight="1">
-      <c r="A20" s="60"/>
+      <c r="A20" s="55"/>
       <c r="B20" s="3">
         <v>31695</v>
       </c>
@@ -3829,7 +3827,7 @@
       </c>
     </row>
     <row r="21" spans="1:10" ht="25.35" customHeight="1">
-      <c r="A21" s="60"/>
+      <c r="A21" s="55"/>
       <c r="B21" s="13">
         <v>31975</v>
       </c>
@@ -3851,56 +3849,56 @@
       </c>
     </row>
     <row r="22" spans="1:10" ht="12.75" customHeight="1">
-      <c r="A22" s="65"/>
-      <c r="B22" s="65"/>
-      <c r="C22" s="65"/>
-      <c r="D22" s="65"/>
-      <c r="E22" s="65"/>
-      <c r="F22" s="65"/>
-      <c r="G22" s="65"/>
-      <c r="H22" s="65"/>
-      <c r="I22" s="65"/>
-      <c r="J22" s="65"/>
+      <c r="A22" s="57"/>
+      <c r="B22" s="57"/>
+      <c r="C22" s="57"/>
+      <c r="D22" s="57"/>
+      <c r="E22" s="57"/>
+      <c r="F22" s="57"/>
+      <c r="G22" s="57"/>
+      <c r="H22" s="57"/>
+      <c r="I22" s="57"/>
+      <c r="J22" s="57"/>
     </row>
     <row r="23" spans="1:10" ht="16.5" customHeight="1">
-      <c r="A23" s="38" t="s">
+      <c r="A23" s="49" t="s">
         <v>57</v>
       </c>
-      <c r="B23" s="39"/>
-      <c r="C23" s="39"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="39"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="39"/>
-      <c r="H23" s="39"/>
-      <c r="I23" s="39"/>
-      <c r="J23" s="40"/>
+      <c r="B23" s="36"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="36"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="36"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="36"/>
+      <c r="J23" s="37"/>
     </row>
     <row r="24" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A24" s="53" t="s">
+      <c r="A24" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="B24" s="43" t="s">
+      <c r="B24" s="40" t="s">
         <v>2</v>
       </c>
       <c r="C24" s="30"/>
-      <c r="D24" s="55" t="s">
+      <c r="D24" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="E24" s="47" t="s">
+      <c r="E24" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="F24" s="48"/>
-      <c r="G24" s="48"/>
-      <c r="H24" s="48"/>
-      <c r="I24" s="48"/>
-      <c r="J24" s="49"/>
+      <c r="F24" s="45"/>
+      <c r="G24" s="45"/>
+      <c r="H24" s="45"/>
+      <c r="I24" s="45"/>
+      <c r="J24" s="46"/>
     </row>
     <row r="25" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A25" s="54"/>
-      <c r="B25" s="44"/>
+      <c r="A25" s="51"/>
+      <c r="B25" s="41"/>
       <c r="C25" s="31"/>
-      <c r="D25" s="56"/>
+      <c r="D25" s="53"/>
       <c r="E25" s="1" t="s">
         <v>5</v>
       </c>
@@ -3921,7 +3919,7 @@
       </c>
     </row>
     <row r="26" spans="1:10" ht="19.7" customHeight="1">
-      <c r="A26" s="63" t="s">
+      <c r="A26" s="54" t="s">
         <v>58</v>
       </c>
       <c r="B26" s="3">
@@ -3947,7 +3945,7 @@
       </c>
     </row>
     <row r="27" spans="1:10" ht="19.7" customHeight="1">
-      <c r="A27" s="60"/>
+      <c r="A27" s="55"/>
       <c r="B27" s="3">
         <v>30743</v>
       </c>
@@ -3971,7 +3969,7 @@
       </c>
     </row>
     <row r="28" spans="1:10" ht="19.7" customHeight="1">
-      <c r="A28" s="60"/>
+      <c r="A28" s="55"/>
       <c r="B28" s="3">
         <v>31048</v>
       </c>
@@ -3993,19 +3991,19 @@
       </c>
     </row>
     <row r="29" spans="1:10" ht="5.25" customHeight="1">
-      <c r="A29" s="59"/>
-      <c r="B29" s="59"/>
-      <c r="C29" s="59"/>
-      <c r="D29" s="59"/>
-      <c r="E29" s="59"/>
-      <c r="F29" s="59"/>
-      <c r="G29" s="59"/>
-      <c r="H29" s="59"/>
-      <c r="I29" s="59"/>
-      <c r="J29" s="59"/>
+      <c r="A29" s="58"/>
+      <c r="B29" s="58"/>
+      <c r="C29" s="58"/>
+      <c r="D29" s="58"/>
+      <c r="E29" s="58"/>
+      <c r="F29" s="58"/>
+      <c r="G29" s="58"/>
+      <c r="H29" s="58"/>
+      <c r="I29" s="58"/>
+      <c r="J29" s="58"/>
     </row>
     <row r="30" spans="1:10" ht="19.7" customHeight="1">
-      <c r="A30" s="60" t="s">
+      <c r="A30" s="55" t="s">
         <v>70</v>
       </c>
       <c r="B30" s="3">
@@ -4029,7 +4027,7 @@
       </c>
     </row>
     <row r="31" spans="1:10" ht="22.35" customHeight="1">
-      <c r="A31" s="60"/>
+      <c r="A31" s="55"/>
       <c r="B31" s="17">
         <v>31041</v>
       </c>
@@ -4051,7 +4049,7 @@
       </c>
     </row>
     <row r="32" spans="1:10" ht="22.35" customHeight="1">
-      <c r="A32" s="61" t="s">
+      <c r="A32" s="59" t="s">
         <v>77</v>
       </c>
       <c r="B32" s="19">
@@ -4077,7 +4075,7 @@
       </c>
     </row>
     <row r="33" spans="1:10" ht="19.7" customHeight="1">
-      <c r="A33" s="61"/>
+      <c r="A33" s="59"/>
       <c r="B33" s="3">
         <v>31235</v>
       </c>
@@ -4099,7 +4097,7 @@
       </c>
     </row>
     <row r="34" spans="1:10" ht="19.7" customHeight="1">
-      <c r="A34" s="61"/>
+      <c r="A34" s="59"/>
       <c r="B34" s="17">
         <v>31042</v>
       </c>
@@ -4122,55 +4120,55 @@
     </row>
     <row r="35" spans="1:10" ht="13.7" customHeight="1">
       <c r="A35" s="21"/>
-      <c r="B35" s="62"/>
-      <c r="C35" s="37"/>
-      <c r="D35" s="37"/>
-      <c r="E35" s="37"/>
-      <c r="F35" s="37"/>
-      <c r="G35" s="37"/>
-      <c r="H35" s="37"/>
-      <c r="I35" s="37"/>
-      <c r="J35" s="37"/>
+      <c r="B35" s="60"/>
+      <c r="C35" s="61"/>
+      <c r="D35" s="61"/>
+      <c r="E35" s="61"/>
+      <c r="F35" s="61"/>
+      <c r="G35" s="61"/>
+      <c r="H35" s="61"/>
+      <c r="I35" s="61"/>
+      <c r="J35" s="61"/>
     </row>
     <row r="36" spans="1:10" ht="17.850000000000001" customHeight="1">
-      <c r="A36" s="38" t="s">
+      <c r="A36" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="B36" s="39"/>
-      <c r="C36" s="39"/>
-      <c r="D36" s="39"/>
-      <c r="E36" s="39"/>
-      <c r="F36" s="39"/>
-      <c r="G36" s="39"/>
-      <c r="H36" s="39"/>
-      <c r="I36" s="39"/>
-      <c r="J36" s="40"/>
+      <c r="B36" s="36"/>
+      <c r="C36" s="36"/>
+      <c r="D36" s="36"/>
+      <c r="E36" s="36"/>
+      <c r="F36" s="36"/>
+      <c r="G36" s="36"/>
+      <c r="H36" s="36"/>
+      <c r="I36" s="36"/>
+      <c r="J36" s="37"/>
     </row>
     <row r="37" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A37" s="53" t="s">
+      <c r="A37" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="B37" s="43" t="s">
+      <c r="B37" s="40" t="s">
         <v>2</v>
       </c>
       <c r="C37" s="30"/>
-      <c r="D37" s="55" t="s">
+      <c r="D37" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="E37" s="47" t="s">
+      <c r="E37" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="F37" s="48"/>
-      <c r="G37" s="48"/>
-      <c r="H37" s="48"/>
-      <c r="I37" s="48"/>
-      <c r="J37" s="49"/>
+      <c r="F37" s="45"/>
+      <c r="G37" s="45"/>
+      <c r="H37" s="45"/>
+      <c r="I37" s="45"/>
+      <c r="J37" s="46"/>
     </row>
     <row r="38" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A38" s="54"/>
-      <c r="B38" s="44"/>
+      <c r="A38" s="51"/>
+      <c r="B38" s="41"/>
       <c r="C38" s="31"/>
-      <c r="D38" s="56"/>
+      <c r="D38" s="53"/>
       <c r="E38" s="1" t="s">
         <v>5</v>
       </c>
@@ -4309,7 +4307,7 @@
       </c>
     </row>
     <row r="44" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A44" s="57"/>
+      <c r="A44" s="34"/>
       <c r="B44" s="22">
         <v>30747</v>
       </c>
@@ -4331,56 +4329,56 @@
       </c>
     </row>
     <row r="45" spans="1:10" ht="16.350000000000001" customHeight="1">
-      <c r="A45" s="58"/>
-      <c r="B45" s="58"/>
-      <c r="C45" s="58"/>
-      <c r="D45" s="58"/>
-      <c r="E45" s="58"/>
-      <c r="F45" s="58"/>
-      <c r="G45" s="58"/>
-      <c r="H45" s="58"/>
-      <c r="I45" s="58"/>
-      <c r="J45" s="58"/>
+      <c r="A45" s="62"/>
+      <c r="B45" s="62"/>
+      <c r="C45" s="62"/>
+      <c r="D45" s="62"/>
+      <c r="E45" s="62"/>
+      <c r="F45" s="62"/>
+      <c r="G45" s="62"/>
+      <c r="H45" s="62"/>
+      <c r="I45" s="62"/>
+      <c r="J45" s="62"/>
     </row>
     <row r="46" spans="1:10" ht="16.5" customHeight="1">
-      <c r="A46" s="38" t="s">
+      <c r="A46" s="49" t="s">
         <v>107</v>
       </c>
-      <c r="B46" s="39"/>
-      <c r="C46" s="39"/>
-      <c r="D46" s="39"/>
-      <c r="E46" s="39"/>
-      <c r="F46" s="39"/>
-      <c r="G46" s="39"/>
-      <c r="H46" s="39"/>
-      <c r="I46" s="39"/>
-      <c r="J46" s="40"/>
+      <c r="B46" s="36"/>
+      <c r="C46" s="36"/>
+      <c r="D46" s="36"/>
+      <c r="E46" s="36"/>
+      <c r="F46" s="36"/>
+      <c r="G46" s="36"/>
+      <c r="H46" s="36"/>
+      <c r="I46" s="36"/>
+      <c r="J46" s="37"/>
     </row>
     <row r="47" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A47" s="53" t="s">
+      <c r="A47" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="B47" s="43" t="s">
+      <c r="B47" s="40" t="s">
         <v>2</v>
       </c>
       <c r="C47" s="30"/>
-      <c r="D47" s="55" t="s">
+      <c r="D47" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="E47" s="47" t="s">
+      <c r="E47" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="F47" s="48"/>
-      <c r="G47" s="48"/>
-      <c r="H47" s="48"/>
-      <c r="I47" s="48"/>
-      <c r="J47" s="49"/>
+      <c r="F47" s="45"/>
+      <c r="G47" s="45"/>
+      <c r="H47" s="45"/>
+      <c r="I47" s="45"/>
+      <c r="J47" s="46"/>
     </row>
     <row r="48" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A48" s="54"/>
-      <c r="B48" s="44"/>
+      <c r="A48" s="51"/>
+      <c r="B48" s="41"/>
       <c r="C48" s="31"/>
-      <c r="D48" s="56"/>
+      <c r="D48" s="53"/>
       <c r="E48" s="1" t="s">
         <v>5</v>
       </c>
@@ -4519,7 +4517,7 @@
       </c>
     </row>
     <row r="54" spans="1:10" ht="60.6" customHeight="1">
-      <c r="A54" s="57"/>
+      <c r="A54" s="34"/>
       <c r="B54" s="23" t="s">
         <v>122</v>
       </c>
@@ -4527,54 +4525,54 @@
       <c r="D54" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="E54" s="50" t="s">
+      <c r="E54" s="63" t="s">
         <v>124</v>
       </c>
-      <c r="F54" s="51"/>
-      <c r="G54" s="51"/>
-      <c r="H54" s="51"/>
-      <c r="I54" s="52"/>
+      <c r="F54" s="64"/>
+      <c r="G54" s="64"/>
+      <c r="H54" s="64"/>
+      <c r="I54" s="65"/>
       <c r="J54" s="24"/>
     </row>
     <row r="55" spans="1:10" ht="18.95" customHeight="1">
-      <c r="A55" s="38" t="s">
+      <c r="A55" s="49" t="s">
         <v>125</v>
       </c>
-      <c r="B55" s="39"/>
-      <c r="C55" s="39"/>
-      <c r="D55" s="39"/>
-      <c r="E55" s="39"/>
-      <c r="F55" s="39"/>
-      <c r="G55" s="39"/>
-      <c r="H55" s="39"/>
-      <c r="I55" s="39"/>
-      <c r="J55" s="40"/>
+      <c r="B55" s="36"/>
+      <c r="C55" s="36"/>
+      <c r="D55" s="36"/>
+      <c r="E55" s="36"/>
+      <c r="F55" s="36"/>
+      <c r="G55" s="36"/>
+      <c r="H55" s="36"/>
+      <c r="I55" s="36"/>
+      <c r="J55" s="37"/>
     </row>
     <row r="56" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A56" s="53" t="s">
+      <c r="A56" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="B56" s="43" t="s">
+      <c r="B56" s="40" t="s">
         <v>2</v>
       </c>
       <c r="C56" s="30"/>
-      <c r="D56" s="55" t="s">
+      <c r="D56" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="E56" s="47" t="s">
+      <c r="E56" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="F56" s="48"/>
-      <c r="G56" s="48"/>
-      <c r="H56" s="48"/>
-      <c r="I56" s="48"/>
-      <c r="J56" s="49"/>
+      <c r="F56" s="45"/>
+      <c r="G56" s="45"/>
+      <c r="H56" s="45"/>
+      <c r="I56" s="45"/>
+      <c r="J56" s="46"/>
     </row>
     <row r="57" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A57" s="54"/>
-      <c r="B57" s="44"/>
+      <c r="A57" s="51"/>
+      <c r="B57" s="41"/>
       <c r="C57" s="31"/>
-      <c r="D57" s="56"/>
+      <c r="D57" s="53"/>
       <c r="E57" s="1" t="s">
         <v>5</v>
       </c>
@@ -4699,66 +4697,66 @@
       <c r="D62" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="E62" s="50" t="s">
+      <c r="E62" s="63" t="s">
         <v>135</v>
       </c>
-      <c r="F62" s="51"/>
-      <c r="G62" s="51"/>
-      <c r="H62" s="51"/>
-      <c r="I62" s="52"/>
+      <c r="F62" s="64"/>
+      <c r="G62" s="64"/>
+      <c r="H62" s="64"/>
+      <c r="I62" s="65"/>
       <c r="J62" s="24"/>
     </row>
     <row r="63" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A63" s="37"/>
-      <c r="B63" s="37"/>
-      <c r="C63" s="37"/>
-      <c r="D63" s="37"/>
-      <c r="E63" s="37"/>
-      <c r="F63" s="37"/>
-      <c r="G63" s="37"/>
-      <c r="H63" s="37"/>
-      <c r="I63" s="37"/>
-      <c r="J63" s="37"/>
+      <c r="A63" s="61"/>
+      <c r="B63" s="61"/>
+      <c r="C63" s="61"/>
+      <c r="D63" s="61"/>
+      <c r="E63" s="61"/>
+      <c r="F63" s="61"/>
+      <c r="G63" s="61"/>
+      <c r="H63" s="61"/>
+      <c r="I63" s="61"/>
+      <c r="J63" s="61"/>
     </row>
     <row r="64" spans="1:10" ht="18.600000000000001" customHeight="1">
-      <c r="A64" s="38" t="s">
+      <c r="A64" s="49" t="s">
         <v>136</v>
       </c>
-      <c r="B64" s="39"/>
-      <c r="C64" s="39"/>
-      <c r="D64" s="39"/>
-      <c r="E64" s="39"/>
-      <c r="F64" s="39"/>
-      <c r="G64" s="39"/>
-      <c r="H64" s="39"/>
-      <c r="I64" s="39"/>
-      <c r="J64" s="40"/>
+      <c r="B64" s="36"/>
+      <c r="C64" s="36"/>
+      <c r="D64" s="36"/>
+      <c r="E64" s="36"/>
+      <c r="F64" s="36"/>
+      <c r="G64" s="36"/>
+      <c r="H64" s="36"/>
+      <c r="I64" s="36"/>
+      <c r="J64" s="37"/>
     </row>
     <row r="65" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A65" s="53" t="s">
+      <c r="A65" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="B65" s="43" t="s">
+      <c r="B65" s="40" t="s">
         <v>2</v>
       </c>
       <c r="C65" s="30"/>
-      <c r="D65" s="55" t="s">
+      <c r="D65" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="E65" s="47" t="s">
+      <c r="E65" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="F65" s="48"/>
-      <c r="G65" s="48"/>
-      <c r="H65" s="48"/>
-      <c r="I65" s="48"/>
-      <c r="J65" s="49"/>
+      <c r="F65" s="45"/>
+      <c r="G65" s="45"/>
+      <c r="H65" s="45"/>
+      <c r="I65" s="45"/>
+      <c r="J65" s="46"/>
     </row>
     <row r="66" spans="1:10" ht="13.7" customHeight="1">
-      <c r="A66" s="54"/>
-      <c r="B66" s="44"/>
+      <c r="A66" s="51"/>
+      <c r="B66" s="41"/>
       <c r="C66" s="31"/>
-      <c r="D66" s="56"/>
+      <c r="D66" s="53"/>
       <c r="E66" s="1" t="s">
         <v>5</v>
       </c>
@@ -4895,56 +4893,56 @@
       </c>
     </row>
     <row r="72" spans="1:10" ht="23.25" customHeight="1">
-      <c r="A72" s="37"/>
-      <c r="B72" s="37"/>
-      <c r="C72" s="37"/>
-      <c r="D72" s="37"/>
-      <c r="E72" s="37"/>
-      <c r="F72" s="37"/>
-      <c r="G72" s="37"/>
-      <c r="H72" s="37"/>
-      <c r="I72" s="37"/>
-      <c r="J72" s="37"/>
+      <c r="A72" s="61"/>
+      <c r="B72" s="61"/>
+      <c r="C72" s="61"/>
+      <c r="D72" s="61"/>
+      <c r="E72" s="61"/>
+      <c r="F72" s="61"/>
+      <c r="G72" s="61"/>
+      <c r="H72" s="61"/>
+      <c r="I72" s="61"/>
+      <c r="J72" s="61"/>
     </row>
     <row r="73" spans="1:10" ht="18.95" customHeight="1">
-      <c r="A73" s="38" t="s">
-        <v>145</v>
-      </c>
-      <c r="B73" s="39"/>
-      <c r="C73" s="39"/>
-      <c r="D73" s="39"/>
-      <c r="E73" s="39"/>
-      <c r="F73" s="39"/>
-      <c r="G73" s="39"/>
-      <c r="H73" s="39"/>
-      <c r="I73" s="39"/>
-      <c r="J73" s="40"/>
+      <c r="A73" s="74" t="s">
+        <v>181</v>
+      </c>
+      <c r="B73" s="36"/>
+      <c r="C73" s="36"/>
+      <c r="D73" s="36"/>
+      <c r="E73" s="36"/>
+      <c r="F73" s="36"/>
+      <c r="G73" s="36"/>
+      <c r="H73" s="36"/>
+      <c r="I73" s="36"/>
+      <c r="J73" s="37"/>
     </row>
     <row r="74" spans="1:10" ht="12.6" customHeight="1">
-      <c r="A74" s="41" t="s">
+      <c r="A74" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B74" s="43" t="s">
+      <c r="B74" s="40" t="s">
         <v>2</v>
       </c>
       <c r="C74" s="30"/>
-      <c r="D74" s="45" t="s">
+      <c r="D74" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="E74" s="47" t="s">
+      <c r="E74" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="F74" s="48"/>
-      <c r="G74" s="48"/>
-      <c r="H74" s="48"/>
-      <c r="I74" s="48"/>
-      <c r="J74" s="49"/>
+      <c r="F74" s="45"/>
+      <c r="G74" s="45"/>
+      <c r="H74" s="45"/>
+      <c r="I74" s="45"/>
+      <c r="J74" s="46"/>
     </row>
     <row r="75" spans="1:10" ht="12.6" customHeight="1">
-      <c r="A75" s="42"/>
-      <c r="B75" s="44"/>
+      <c r="A75" s="39"/>
+      <c r="B75" s="41"/>
       <c r="C75" s="31"/>
-      <c r="D75" s="46"/>
+      <c r="D75" s="43"/>
       <c r="E75" s="1" t="s">
         <v>5</v>
       </c>
@@ -4973,21 +4971,21 @@
       </c>
       <c r="C76" s="3"/>
       <c r="D76" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="E76" s="5" t="s">
         <v>146</v>
-      </c>
-      <c r="E76" s="5" t="s">
-        <v>147</v>
       </c>
       <c r="F76" s="6"/>
       <c r="G76" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H76" s="6"/>
       <c r="I76" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="J76" s="7" t="s">
         <v>147</v>
-      </c>
-      <c r="J76" s="7" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="77" spans="1:10" ht="20.85" customHeight="1">
@@ -4997,18 +4995,18 @@
       </c>
       <c r="C77" s="3"/>
       <c r="D77" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="E77" s="5" t="s">
         <v>149</v>
-      </c>
-      <c r="E77" s="5" t="s">
-        <v>150</v>
       </c>
       <c r="F77" s="6"/>
       <c r="G77" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H77" s="6"/>
       <c r="I77" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J77" s="7" t="s">
         <v>106</v>
@@ -5021,18 +5019,18 @@
       </c>
       <c r="C78" s="3"/>
       <c r="D78" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="E78" s="5" t="s">
         <v>151</v>
-      </c>
-      <c r="E78" s="5" t="s">
-        <v>152</v>
       </c>
       <c r="F78" s="6"/>
       <c r="G78" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H78" s="6"/>
       <c r="I78" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="J78" s="7" t="s">
         <v>130</v>
@@ -5045,19 +5043,19 @@
       </c>
       <c r="C79" s="3"/>
       <c r="D79" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E79" s="6"/>
       <c r="F79" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G79" s="6"/>
       <c r="H79" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I79" s="6"/>
       <c r="J79" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="80" spans="1:10" ht="20.85" customHeight="1">
@@ -5067,7 +5065,7 @@
       </c>
       <c r="C80" s="3"/>
       <c r="D80" s="8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E80" s="6"/>
       <c r="F80" s="5" t="s">
@@ -5079,48 +5077,48 @@
       </c>
       <c r="I80" s="6"/>
       <c r="J80" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="82" spans="1:10" ht="15">
-      <c r="A82" s="73" t="s">
-        <v>181</v>
-      </c>
-      <c r="B82" s="39"/>
-      <c r="C82" s="39"/>
-      <c r="D82" s="39"/>
-      <c r="E82" s="39"/>
-      <c r="F82" s="39"/>
-      <c r="G82" s="39"/>
-      <c r="H82" s="39"/>
-      <c r="I82" s="39"/>
-      <c r="J82" s="40"/>
+      <c r="A82" s="35" t="s">
+        <v>182</v>
+      </c>
+      <c r="B82" s="36"/>
+      <c r="C82" s="36"/>
+      <c r="D82" s="36"/>
+      <c r="E82" s="36"/>
+      <c r="F82" s="36"/>
+      <c r="G82" s="36"/>
+      <c r="H82" s="36"/>
+      <c r="I82" s="36"/>
+      <c r="J82" s="37"/>
     </row>
     <row r="83" spans="1:10">
-      <c r="A83" s="41" t="s">
+      <c r="A83" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B83" s="43" t="s">
+      <c r="B83" s="40" t="s">
         <v>2</v>
       </c>
       <c r="C83" s="30"/>
-      <c r="D83" s="45" t="s">
+      <c r="D83" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="E83" s="47" t="s">
+      <c r="E83" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="F83" s="48"/>
-      <c r="G83" s="48"/>
-      <c r="H83" s="48"/>
-      <c r="I83" s="48"/>
-      <c r="J83" s="49"/>
+      <c r="F83" s="45"/>
+      <c r="G83" s="45"/>
+      <c r="H83" s="45"/>
+      <c r="I83" s="45"/>
+      <c r="J83" s="46"/>
     </row>
     <row r="84" spans="1:10">
-      <c r="A84" s="42"/>
-      <c r="B84" s="44"/>
+      <c r="A84" s="39"/>
+      <c r="B84" s="41"/>
       <c r="C84" s="31"/>
-      <c r="D84" s="46"/>
+      <c r="D84" s="43"/>
       <c r="E84" s="1" t="s">
         <v>5</v>
       </c>
@@ -5149,21 +5147,21 @@
       </c>
       <c r="C85" s="3"/>
       <c r="D85" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E85" s="6"/>
       <c r="F85" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="G85" s="5" t="s">
         <v>159</v>
-      </c>
-      <c r="G85" s="5" t="s">
-        <v>160</v>
       </c>
       <c r="H85" s="6"/>
       <c r="I85" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="J85" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="86" spans="1:10" ht="27">
@@ -5173,21 +5171,21 @@
       </c>
       <c r="C86" s="3"/>
       <c r="D86" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F86" s="6"/>
       <c r="G86" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H86" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I86" s="6"/>
       <c r="J86" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="87" spans="1:10" ht="27">
@@ -5197,91 +5195,45 @@
       </c>
       <c r="C87" s="3"/>
       <c r="D87" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="E87" s="5" t="s">
         <v>162</v>
-      </c>
-      <c r="E87" s="5" t="s">
-        <v>163</v>
       </c>
       <c r="F87" s="6"/>
       <c r="G87" s="6"/>
       <c r="H87" s="6"/>
       <c r="I87" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J87" s="7" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="88" spans="1:10" ht="27">
-      <c r="A88" s="57"/>
+      <c r="A88" s="34"/>
       <c r="B88" s="3">
         <v>31272</v>
       </c>
       <c r="C88" s="3"/>
       <c r="D88" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E88" s="6"/>
       <c r="F88" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G88" s="6"/>
       <c r="H88" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="I88" s="6"/>
       <c r="J88" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="62">
-    <mergeCell ref="A85:A88"/>
-    <mergeCell ref="A82:J82"/>
-    <mergeCell ref="A83:A84"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="D83:D84"/>
-    <mergeCell ref="E83:J83"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="A7:A13"/>
-    <mergeCell ref="A15:A21"/>
-    <mergeCell ref="A22:J22"/>
-    <mergeCell ref="A23:J23"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="E24:J24"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="A29:J29"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="A32:A34"/>
-    <mergeCell ref="B35:J35"/>
-    <mergeCell ref="A36:J36"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="E37:J37"/>
-    <mergeCell ref="A39:A44"/>
-    <mergeCell ref="A45:J45"/>
-    <mergeCell ref="A46:J46"/>
-    <mergeCell ref="A47:A48"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="D47:D48"/>
-    <mergeCell ref="E47:J47"/>
-    <mergeCell ref="D65:D66"/>
-    <mergeCell ref="E65:J65"/>
-    <mergeCell ref="A49:A54"/>
-    <mergeCell ref="E54:I54"/>
-    <mergeCell ref="A55:J55"/>
-    <mergeCell ref="A56:A57"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="D56:D57"/>
-    <mergeCell ref="E56:J56"/>
     <mergeCell ref="A76:A80"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
@@ -5298,6 +5250,52 @@
     <mergeCell ref="A64:J64"/>
     <mergeCell ref="A65:A66"/>
     <mergeCell ref="B65:B66"/>
+    <mergeCell ref="D65:D66"/>
+    <mergeCell ref="E65:J65"/>
+    <mergeCell ref="A49:A54"/>
+    <mergeCell ref="E54:I54"/>
+    <mergeCell ref="A55:J55"/>
+    <mergeCell ref="A56:A57"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="E56:J56"/>
+    <mergeCell ref="A39:A44"/>
+    <mergeCell ref="A45:J45"/>
+    <mergeCell ref="A46:J46"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="D47:D48"/>
+    <mergeCell ref="E47:J47"/>
+    <mergeCell ref="A36:J36"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="E37:J37"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="B35:J35"/>
+    <mergeCell ref="A7:A13"/>
+    <mergeCell ref="A15:A21"/>
+    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="A23:J23"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:J24"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="A85:A88"/>
+    <mergeCell ref="A82:J82"/>
+    <mergeCell ref="A83:A84"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="D83:D84"/>
+    <mergeCell ref="E83:J83"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5321,32 +5319,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21.75" customHeight="1">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="69" t="s">
+        <v>178</v>
+      </c>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75">
+      <c r="A2" s="71" t="s">
         <v>179</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-    </row>
-    <row r="2" spans="1:10" ht="15.75">
-      <c r="A2" s="70" t="s">
-        <v>180</v>
-      </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
     </row>
     <row r="3" spans="1:10" ht="24.75" customHeight="1"/>
     <row r="4" spans="1:10" ht="12.6" customHeight="1"/>
@@ -5356,55 +5354,55 @@
     <row r="8" spans="1:10" ht="20.85" customHeight="1"/>
     <row r="9" spans="1:10" ht="20.85" customHeight="1"/>
     <row r="10" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A10" s="58"/>
-      <c r="B10" s="58"/>
-      <c r="C10" s="58"/>
-      <c r="D10" s="58"/>
-      <c r="E10" s="58"/>
-      <c r="F10" s="58"/>
-      <c r="G10" s="58"/>
-      <c r="H10" s="58"/>
-      <c r="I10" s="58"/>
-      <c r="J10" s="58"/>
+      <c r="A10" s="62"/>
+      <c r="B10" s="62"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
+      <c r="G10" s="62"/>
+      <c r="H10" s="62"/>
+      <c r="I10" s="62"/>
+      <c r="J10" s="62"/>
     </row>
     <row r="11" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A11" s="38" t="s">
+      <c r="A11" s="49" t="s">
+        <v>166</v>
+      </c>
+      <c r="B11" s="36"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="36"/>
+      <c r="E11" s="36"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="36"/>
+      <c r="H11" s="36"/>
+      <c r="I11" s="36"/>
+      <c r="J11" s="37"/>
+    </row>
+    <row r="12" spans="1:10" ht="12.6" customHeight="1">
+      <c r="A12" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C12" s="72"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="44" t="s">
+        <v>4</v>
+      </c>
+      <c r="F12" s="45"/>
+      <c r="G12" s="45"/>
+      <c r="H12" s="45"/>
+      <c r="I12" s="45"/>
+      <c r="J12" s="46"/>
+    </row>
+    <row r="13" spans="1:10" ht="12.6" customHeight="1">
+      <c r="A13" s="39"/>
+      <c r="B13" s="41"/>
+      <c r="C13" s="73"/>
+      <c r="D13" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="B11" s="39"/>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="39"/>
-      <c r="I11" s="39"/>
-      <c r="J11" s="40"/>
-    </row>
-    <row r="12" spans="1:10" ht="12.6" customHeight="1">
-      <c r="A12" s="41" t="s">
-        <v>1</v>
-      </c>
-      <c r="B12" s="43" t="s">
-        <v>2</v>
-      </c>
-      <c r="C12" s="71"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="47" t="s">
-        <v>4</v>
-      </c>
-      <c r="F12" s="48"/>
-      <c r="G12" s="48"/>
-      <c r="H12" s="48"/>
-      <c r="I12" s="48"/>
-      <c r="J12" s="49"/>
-    </row>
-    <row r="13" spans="1:10" ht="12.6" customHeight="1">
-      <c r="A13" s="42"/>
-      <c r="B13" s="44"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="1" t="s">
-        <v>168</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>5</v>
@@ -5433,7 +5431,7 @@
         <v>30809</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D14" s="26">
         <v>24</v>
@@ -5444,7 +5442,7 @@
       <c r="H14" s="15"/>
       <c r="I14" s="15"/>
       <c r="J14" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="12.2" customHeight="1">
@@ -5453,7 +5451,7 @@
         <v>32404</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D15" s="26">
         <v>2</v>
@@ -5473,7 +5471,7 @@
         <v>32405</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D16" s="26">
         <v>1</v>
@@ -5484,7 +5482,7 @@
       <c r="H16" s="15"/>
       <c r="I16" s="15"/>
       <c r="J16" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="12.2" customHeight="1">
@@ -5493,7 +5491,7 @@
         <v>32406</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D17" s="26">
         <v>3</v>
@@ -5513,7 +5511,7 @@
         <v>32407</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D18" s="26">
         <v>2</v>
@@ -5524,7 +5522,7 @@
       <c r="H18" s="15"/>
       <c r="I18" s="15"/>
       <c r="J18" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="12.2" customHeight="1">
@@ -5533,7 +5531,7 @@
         <v>32408</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D19" s="26">
         <v>2</v>
@@ -5553,7 +5551,7 @@
         <v>32409</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D20" s="26">
         <v>1</v>
@@ -5573,7 +5571,7 @@
         <v>32410</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D21" s="26">
         <v>5</v>
@@ -5584,7 +5582,7 @@
       <c r="H21" s="15"/>
       <c r="I21" s="15"/>
       <c r="J21" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="12.2" customHeight="1">
@@ -5593,7 +5591,7 @@
         <v>32411</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D22" s="26">
         <v>5</v>
@@ -5604,7 +5602,7 @@
       <c r="H22" s="15"/>
       <c r="I22" s="15"/>
       <c r="J22" s="7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="12.2" customHeight="1">
@@ -5613,7 +5611,7 @@
         <v>32412</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D23" s="26">
         <v>2</v>
@@ -5624,7 +5622,7 @@
       <c r="H23" s="15"/>
       <c r="I23" s="15"/>
       <c r="J23" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="12.2" customHeight="1">
@@ -5633,7 +5631,7 @@
         <v>32413</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D24" s="26">
         <v>1</v>
@@ -5653,7 +5651,7 @@
         <v>32414</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D25" s="26">
         <v>24</v>
@@ -5664,16 +5662,16 @@
       <c r="H25" s="15"/>
       <c r="I25" s="15"/>
       <c r="J25" s="7" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A26" s="57"/>
+      <c r="A26" s="34"/>
       <c r="B26" s="13">
         <v>32345</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D26" s="26">
         <v>23</v>

</xml_diff>